<commit_message>
Verificaciones de campos y ejemplos
</commit_message>
<xml_diff>
--- a/database/seeders/data/05_FINANZAS.xlsx
+++ b/database/seeders/data/05_FINANZAS.xlsx
@@ -2,19 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SALDOS INICIALES" sheetId="1" r:id="Rf2943bf156634cc0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CARGOS" sheetId="2" r:id="R352062916a524d57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PAGOS" sheetId="3" r:id="R7103ad88ae0b492a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="APLICACIONES DE PAGOS" sheetId="4" r:id="R275bd32f6bd94d0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SALDOS A FAVOR" sheetId="5" r:id="R5da1017849bd46c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MOVIMIENTOS DE SALDO" sheetId="6" r:id="R3fb1ebb380c74eb7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NOTAS DE COBRANZA" sheetId="7" r:id="R175abf2413ea4803"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OPERACIONES SPEI" sheetId="8" r:id="R83ca64acfd234ff5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="APLICACIONES SPEI" sheetId="9" r:id="R214cb87ae8f6424a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FUENTES DE PAGO" sheetId="10" r:id="R4cfa026be2164810"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CORTES DE CAJA" sheetId="11" r:id="R9c2b3e07f3424456"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DESGLOSE DE EFECTIVO" sheetId="12" r:id="Reb09415657334c17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CORTES GLOBALES" sheetId="13" r:id="R196e3c05a11f4dcf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SALDOS INICIALES" sheetId="1" r:id="Rde6f91b221a14471"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CARGOS" sheetId="2" r:id="Rbe354f0eb48e49b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PAGOS" sheetId="3" r:id="R9bc46b6caa844cf1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="APLICACIONES DE PAGOS" sheetId="4" r:id="Rf7ec109c5c48468e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SALDOS A FAVOR" sheetId="5" r:id="R7cfb32b292f2454a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MOVIMIENTOS DE SALDO" sheetId="6" r:id="R920f250e57744df0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NOTAS DE COBRANZA" sheetId="7" r:id="R826e1767126c4964"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OPERACIONES SPEI" sheetId="8" r:id="Rffd419052316499f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="APLICACIONES SPEI" sheetId="9" r:id="Rf603e04dec604fd7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FUENTES DE PAGO" sheetId="10" r:id="Rfd01b108383f4abd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CORTES DE CAJA" sheetId="11" r:id="R361e165dd1634679"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DESGLOSE DE EFECTIVO" sheetId="12" r:id="R2626a63198974c2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CORTES GLOBALES" sheetId="13" r:id="Rca5c05c21a964cfc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INSTRUCCIONES" sheetId="14" r:id="R32076989c8cb419e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EJEMPLOS" sheetId="15" r:id="R8404f5357f5645e7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -25,7 +27,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="3">
+  <x:numFmts count="3">
+    <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
+    <x:numFmt numFmtId="201" formatCode="&quot;$&quot;#,##0.00"/>
+    <x:numFmt numFmtId="202" formatCode="yyyy-mm-dd hh:mm"/>
+  </x:numFmts>
+  <x:fonts count="10">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -41,8 +48,47 @@
       <x:color rgb="FF222222"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="14"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFC0392B"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF2980B9"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF1E8449"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="18">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -54,8 +100,83 @@
         <x:fgColor rgb="FF1F4E78"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFC0392B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2980B9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1A252F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFADBD8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD6EAF8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD5F5E3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEBF5FB"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1A252F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFC0392B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2980B9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEBF5FB"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1A252F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFC0392B"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2980B9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEBF5FB"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="2">
+  <x:borders count="3">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -71,11 +192,25 @@
         <x:color rgb="FFFFFFFF"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9D9D9"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9D9D9"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9D9D9"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9D9D9"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="9">
+  <x:cellXfs count="105">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -92,6 +227,204 @@
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="6" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="6" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="16" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="17" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="17" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="17" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="17" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="6" fillId="17" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="6" fillId="17" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -308,25 +641,25 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
-      <x:c r="A1" s="6" t="str">
+      <x:c r="A1" s="10" t="str">
         <x:v>FECHA DE CORTE</x:v>
       </x:c>
-      <x:c r="B1" s="6" t="str">
+      <x:c r="B1" s="10" t="str">
         <x:v>NÚMERO DE MEMBRESÍA</x:v>
       </x:c>
-      <x:c r="C1" s="6" t="str">
+      <x:c r="C1" s="10" t="str">
         <x:v>NOMBRE DEL CLUB</x:v>
       </x:c>
-      <x:c r="D1" s="6" t="str">
+      <x:c r="D1" s="12" t="str">
         <x:v>SALDO TOTAL PENDIENTE</x:v>
       </x:c>
-      <x:c r="E1" s="6" t="str">
+      <x:c r="E1" s="12" t="str">
         <x:v>SALDO VENCIDO</x:v>
       </x:c>
-      <x:c r="F1" s="6" t="str">
+      <x:c r="F1" s="12" t="str">
         <x:v>SALDO A FAVOR</x:v>
       </x:c>
-      <x:c r="G1" s="6" t="str">
+      <x:c r="G1" s="12" t="str">
         <x:v>NOTAS</x:v>
       </x:c>
     </x:row>
@@ -2150,46 +2483,46 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
-      <x:c r="A1" s="6" t="str">
+      <x:c r="A1" s="10" t="str">
         <x:v>NÚMERO DE SOCIO</x:v>
       </x:c>
-      <x:c r="B1" s="6" t="str">
+      <x:c r="B1" s="12" t="str">
         <x:v>NOMBRE</x:v>
       </x:c>
-      <x:c r="C1" s="6" t="str">
+      <x:c r="C1" s="12" t="str">
         <x:v>APELLIDO PATERNO</x:v>
       </x:c>
-      <x:c r="D1" s="6" t="str">
+      <x:c r="D1" s="12" t="str">
         <x:v>APELLIDO MATERNO</x:v>
       </x:c>
-      <x:c r="E1" s="6" t="str">
+      <x:c r="E1" s="10" t="str">
         <x:v>NOMBRE DEL CLUB</x:v>
       </x:c>
-      <x:c r="F1" s="6" t="str">
+      <x:c r="F1" s="12" t="str">
         <x:v>IDENTIFICADOR DE LA TARJETA EN EL PROVEEDOR</x:v>
       </x:c>
-      <x:c r="G1" s="6" t="str">
+      <x:c r="G1" s="12" t="str">
         <x:v>TIPO DE TARJETA</x:v>
       </x:c>
-      <x:c r="H1" s="6" t="str">
+      <x:c r="H1" s="12" t="str">
         <x:v>ÚLTIMOS CUATRO DÍGITOS</x:v>
       </x:c>
-      <x:c r="I1" s="6" t="str">
+      <x:c r="I1" s="12" t="str">
         <x:v>MARCA DE LA TARJETA</x:v>
       </x:c>
-      <x:c r="J1" s="6" t="str">
+      <x:c r="J1" s="12" t="str">
         <x:v>MES DE VENCIMIENTO</x:v>
       </x:c>
-      <x:c r="K1" s="6" t="str">
+      <x:c r="K1" s="12" t="str">
         <x:v>AÑO DE VENCIMIENTO</x:v>
       </x:c>
-      <x:c r="L1" s="6" t="str">
+      <x:c r="L1" s="12" t="str">
         <x:v>NOMBRE DEL TITULAR DE LA TARJETA</x:v>
       </x:c>
-      <x:c r="M1" s="6" t="str">
+      <x:c r="M1" s="12" t="str">
         <x:v>ES LA TARJETA PREDETERMINADA</x:v>
       </x:c>
-      <x:c r="N1" s="6" t="str">
+      <x:c r="N1" s="12" t="str">
         <x:v>FECHA DE BAJA</x:v>
       </x:c>
     </x:row>
@@ -5406,46 +5739,46 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
-      <x:c r="A1" s="6" t="str">
+      <x:c r="A1" s="10" t="str">
         <x:v>FOLIO O REFERENCIA DEL CORTE ANTERIOR</x:v>
       </x:c>
-      <x:c r="B1" s="6" t="str">
+      <x:c r="B1" s="10" t="str">
         <x:v>NOMBRE DEL CLUB</x:v>
       </x:c>
-      <x:c r="C1" s="6" t="str">
+      <x:c r="C1" s="12" t="str">
         <x:v>NOMBRE DEL CAJERO</x:v>
       </x:c>
-      <x:c r="D1" s="6" t="str">
+      <x:c r="D1" s="12" t="str">
         <x:v>CORREO DEL CAJERO</x:v>
       </x:c>
-      <x:c r="E1" s="6" t="str">
+      <x:c r="E1" s="10" t="str">
         <x:v>FECHA DEL CORTE</x:v>
       </x:c>
-      <x:c r="F1" s="6" t="str">
+      <x:c r="F1" s="12" t="str">
         <x:v>FONDO INICIAL</x:v>
       </x:c>
-      <x:c r="G1" s="6" t="str">
+      <x:c r="G1" s="10" t="str">
         <x:v>ESTATUS</x:v>
       </x:c>
-      <x:c r="H1" s="6" t="str">
+      <x:c r="H1" s="12" t="str">
         <x:v>FECHA Y HORA DE APERTURA</x:v>
       </x:c>
-      <x:c r="I1" s="6" t="str">
+      <x:c r="I1" s="12" t="str">
         <x:v>FECHA Y HORA DE CIERRE</x:v>
       </x:c>
-      <x:c r="J1" s="6" t="str">
+      <x:c r="J1" s="12" t="str">
         <x:v>EFECTIVO CONTADO</x:v>
       </x:c>
-      <x:c r="K1" s="6" t="str">
+      <x:c r="K1" s="12" t="str">
         <x:v>EFECTIVO ESPERADO</x:v>
       </x:c>
-      <x:c r="L1" s="6" t="str">
+      <x:c r="L1" s="12" t="str">
         <x:v>DIFERENCIA DE EFECTIVO</x:v>
       </x:c>
-      <x:c r="M1" s="6" t="str">
+      <x:c r="M1" s="10" t="str">
         <x:v>FOLIO O REFERENCIA DEL CORTE GLOBAL</x:v>
       </x:c>
-      <x:c r="N1" s="6" t="str">
+      <x:c r="N1" s="12" t="str">
         <x:v>NOTAS</x:v>
       </x:c>
     </x:row>
@@ -8655,25 +8988,25 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
-      <x:c r="A1" s="6" t="str">
+      <x:c r="A1" s="10" t="str">
         <x:v>FOLIO O REFERENCIA DEL CORTE ANTERIOR</x:v>
       </x:c>
-      <x:c r="B1" s="6" t="str">
+      <x:c r="B1" s="10" t="str">
         <x:v>NOMBRE DEL CLUB</x:v>
       </x:c>
-      <x:c r="C1" s="6" t="str">
+      <x:c r="C1" s="12" t="str">
         <x:v>CORREO DEL CAJERO</x:v>
       </x:c>
-      <x:c r="D1" s="6" t="str">
+      <x:c r="D1" s="12" t="str">
         <x:v>FECHA Y HORA DE APERTURA</x:v>
       </x:c>
-      <x:c r="E1" s="6" t="str">
+      <x:c r="E1" s="12" t="str">
         <x:v>DENOMINACIÓN</x:v>
       </x:c>
-      <x:c r="F1" s="6" t="str">
+      <x:c r="F1" s="12" t="str">
         <x:v>CANTIDAD</x:v>
       </x:c>
-      <x:c r="G1" s="6" t="str">
+      <x:c r="G1" s="12" t="str">
         <x:v>SUBTOTAL</x:v>
       </x:c>
     </x:row>
@@ -10490,25 +10823,25 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
-      <x:c r="A1" s="6" t="str">
+      <x:c r="A1" s="10" t="str">
         <x:v>FOLIO O REFERENCIA DEL CORTE GLOBAL</x:v>
       </x:c>
-      <x:c r="B1" s="6" t="str">
+      <x:c r="B1" s="10" t="str">
         <x:v>NOMBRE DEL CLUB</x:v>
       </x:c>
-      <x:c r="C1" s="6" t="str">
+      <x:c r="C1" s="10" t="str">
         <x:v>FECHA DEL CORTE</x:v>
       </x:c>
-      <x:c r="D1" s="6" t="str">
+      <x:c r="D1" s="10" t="str">
         <x:v>ESTATUS</x:v>
       </x:c>
-      <x:c r="E1" s="6" t="str">
+      <x:c r="E1" s="12" t="str">
         <x:v>CORREO DE QUIEN CREÓ EL CORTE</x:v>
       </x:c>
-      <x:c r="F1" s="6" t="str">
+      <x:c r="F1" s="12" t="str">
         <x:v>FECHA Y HORA DE CIERRE</x:v>
       </x:c>
-      <x:c r="G1" s="6" t="str">
+      <x:c r="G1" s="12" t="str">
         <x:v>NOTAS</x:v>
       </x:c>
     </x:row>
@@ -12304,6 +12637,2372 @@
       <x:c r="G200" s="8"/>
     </x:row>
   </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF1A252F"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="76" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="4" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="34" t="str">
+        <x:v>INSTRUCCIONES DE CAPTURA</x:v>
+      </x:c>
+      <x:c r="B1" s="34"/>
+      <x:c r="C1" s="34"/>
+    </x:row>
+    <x:row r="2" ht="24" customHeight="1">
+      <x:c r="A2" s="35"/>
+      <x:c r="B2" s="35"/>
+      <x:c r="C2" s="35"/>
+    </x:row>
+    <x:row r="3" ht="24" customHeight="1">
+      <x:c r="A3" s="36" t="str">
+        <x:v>REGLAS GENERALES</x:v>
+      </x:c>
+      <x:c r="B3" s="36"/>
+      <x:c r="C3" s="36"/>
+    </x:row>
+    <x:row r="4" ht="24" customHeight="1">
+      <x:c r="A4" s="37" t="str">
+        <x:v>ENCABEZADOS</x:v>
+      </x:c>
+      <x:c r="B4" s="38" t="str">
+        <x:v>No modificar los encabezados de las hojas de captura.</x:v>
+      </x:c>
+      <x:c r="C4" s="38"/>
+    </x:row>
+    <x:row r="5" ht="24" customHeight="1">
+      <x:c r="A5" s="37" t="str">
+        <x:v>FECHAS</x:v>
+      </x:c>
+      <x:c r="B5" s="38" t="str">
+        <x:v>Usar formato AAAA-MM-DD. Para fecha y hora: AAAA-MM-DD HH:MM.</x:v>
+      </x:c>
+      <x:c r="C5" s="38"/>
+    </x:row>
+    <x:row r="6" ht="24" customHeight="1">
+      <x:c r="A6" s="37" t="str">
+        <x:v>DATOS DESCONOCIDOS</x:v>
+      </x:c>
+      <x:c r="B6" s="38" t="str">
+        <x:v>Dejar la celda vacía cuando no se cuente con el dato.</x:v>
+      </x:c>
+      <x:c r="C6" s="38"/>
+    </x:row>
+    <x:row r="7" ht="24" customHeight="1">
+      <x:c r="A7" s="37" t="str">
+        <x:v>REFERENCIAS</x:v>
+      </x:c>
+      <x:c r="B7" s="38" t="str">
+        <x:v>Repetir nombre, número de socio, membresía o folio; no usar IDs internos.</x:v>
+      </x:c>
+      <x:c r="C7" s="38"/>
+    </x:row>
+    <x:row r="8" ht="24" customHeight="1">
+      <x:c r="A8" s="37" t="str">
+        <x:v>EJEMPLOS</x:v>
+      </x:c>
+      <x:c r="B8" s="38" t="str">
+        <x:v>La hoja EJEMPLOS es solo guía y no se debe importar como información real.</x:v>
+      </x:c>
+      <x:c r="C8" s="38"/>
+    </x:row>
+    <x:row r="9" ht="24" customHeight="1">
+      <x:c r="A9" s="35"/>
+      <x:c r="B9" s="35"/>
+      <x:c r="C9" s="35"/>
+    </x:row>
+    <x:row r="10" ht="24" customHeight="1">
+      <x:c r="A10" s="36" t="str">
+        <x:v>LEYENDA DE COLORES</x:v>
+      </x:c>
+      <x:c r="B10" s="36"/>
+      <x:c r="C10" s="36"/>
+    </x:row>
+    <x:row r="11" ht="24" customHeight="1">
+      <x:c r="A11" s="39" t="str">
+        <x:v>ENCABEZADO ROJO</x:v>
+      </x:c>
+      <x:c r="B11" s="39" t="str">
+        <x:v>Campo básico para identificar o registrar el dato.</x:v>
+      </x:c>
+      <x:c r="C11" s="39"/>
+    </x:row>
+    <x:row r="12" ht="24" customHeight="1">
+      <x:c r="A12" s="40" t="str">
+        <x:v>ENCABEZADO AZUL</x:v>
+      </x:c>
+      <x:c r="B12" s="40" t="str">
+        <x:v>Campo opcional; llenar cuando se cuente con la información.</x:v>
+      </x:c>
+      <x:c r="C12" s="40"/>
+    </x:row>
+    <x:row r="13" ht="24" customHeight="1">
+      <x:c r="A13" s="41" t="str">
+        <x:v>ENCABEZADO VERDE</x:v>
+      </x:c>
+      <x:c r="B13" s="41" t="str">
+        <x:v>Catálogo de consulta o solo lectura. No modificar.</x:v>
+      </x:c>
+      <x:c r="C13" s="41"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:C1"/>
+    <x:mergeCell ref="A3:C3"/>
+    <x:mergeCell ref="A10:C10"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF1A252F"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="22" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="22" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="22" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="22" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="22" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="22" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="22" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="22" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="22" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="22" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="22" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="22" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="22" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="22" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="22" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="22" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="24" customHeight="1">
+      <x:c r="A1" s="84" t="str">
+        <x:v>EJEMPLOS: SALDOS INICIALES</x:v>
+      </x:c>
+      <x:c r="B1" s="84"/>
+      <x:c r="C1" s="84"/>
+      <x:c r="D1" s="84"/>
+      <x:c r="E1" s="84"/>
+      <x:c r="F1" s="84"/>
+      <x:c r="G1" s="84"/>
+    </x:row>
+    <x:row r="2" ht="42" customHeight="1">
+      <x:c r="A2" s="90" t="str">
+        <x:v>FECHA DE CORTE</x:v>
+      </x:c>
+      <x:c r="B2" s="90" t="str">
+        <x:v>NÚMERO DE MEMBRESÍA</x:v>
+      </x:c>
+      <x:c r="C2" s="90" t="str">
+        <x:v>NOMBRE DEL CLUB</x:v>
+      </x:c>
+      <x:c r="D2" s="96" t="str">
+        <x:v>SALDO TOTAL PENDIENTE</x:v>
+      </x:c>
+      <x:c r="E2" s="96" t="str">
+        <x:v>SALDO VENCIDO</x:v>
+      </x:c>
+      <x:c r="F2" s="96" t="str">
+        <x:v>SALDO A FAVOR</x:v>
+      </x:c>
+      <x:c r="G2" s="96" t="str">
+        <x:v>NOTAS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="24" customHeight="1">
+      <x:c r="A3" s="102" t="n">
+        <x:v>46037</x:v>
+      </x:c>
+      <x:c r="B3" s="101" t="str">
+        <x:v>M-1001</x:v>
+      </x:c>
+      <x:c r="C3" s="101" t="str">
+        <x:v>PARQUE ESPAÑA</x:v>
+      </x:c>
+      <x:c r="D3" s="103" t="n">
+        <x:v>2500</x:v>
+      </x:c>
+      <x:c r="E3" s="103" t="n">
+        <x:v>2500</x:v>
+      </x:c>
+      <x:c r="F3" s="103" t="n">
+        <x:v>2500</x:v>
+      </x:c>
+      <x:c r="G3" s="101" t="str">
+        <x:v>Registro de ejemplo para el socio 1001.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="24" customHeight="1">
+      <x:c r="A4" s="102" t="n">
+        <x:v>46044.291666666664</x:v>
+      </x:c>
+      <x:c r="B4" s="101" t="str">
+        <x:v>M-1002</x:v>
+      </x:c>
+      <x:c r="C4" s="101" t="str">
+        <x:v>PARQUE ESPAÑA</x:v>
+      </x:c>
+      <x:c r="D4" s="103" t="n">
+        <x:v>850</x:v>
+      </x:c>
+      <x:c r="E4" s="103" t="n">
+        <x:v>850</x:v>
+      </x:c>
+      <x:c r="F4" s="103" t="n">
+        <x:v>850</x:v>
+      </x:c>
+      <x:c r="G4" s="101" t="str">
+        <x:v>Registro de ejemplo para el socio 1002.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="24" customHeight="1">
+      <x:c r="A5" s="102" t="n">
+        <x:v>46051.333333333336</x:v>
+      </x:c>
+      <x:c r="B5" s="101" t="str">
+        <x:v>M-1003</x:v>
+      </x:c>
+      <x:c r="C5" s="101" t="str">
+        <x:v>PARQUE ESPAÑA</x:v>
+      </x:c>
+      <x:c r="D5" s="103" t="n">
+        <x:v>1200</x:v>
+      </x:c>
+      <x:c r="E5" s="103" t="n">
+        <x:v>1200</x:v>
+      </x:c>
+      <x:c r="F5" s="103" t="n">
+        <x:v>1200</x:v>
+      </x:c>
+      <x:c r="G5" s="101" t="str">
+        <x:v>Registro de ejemplo para el socio 1003.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="24" customHeight="1">
+      <x:c r="A6"/>
+      <x:c r="B6"/>
+      <x:c r="C6"/>
+      <x:c r="D6"/>
+      <x:c r="E6"/>
+      <x:c r="F6"/>
+      <x:c r="G6"/>
+      <x:c r="H6"/>
+      <x:c r="I6"/>
+      <x:c r="J6"/>
+      <x:c r="K6"/>
+      <x:c r="L6"/>
+      <x:c r="M6"/>
+      <x:c r="N6"/>
+      <x:c r="O6"/>
+      <x:c r="P6"/>
+      <x:c r="Q6"/>
+      <x:c r="R6"/>
+      <x:c r="S6"/>
+      <x:c r="T6"/>
+      <x:c r="U6"/>
+      <x:c r="V6"/>
+    </x:row>
+    <x:row r="7" ht="42" customHeight="1">
+      <x:c r="A7"/>
+      <x:c r="B7"/>
+      <x:c r="C7"/>
+      <x:c r="D7"/>
+      <x:c r="E7"/>
+      <x:c r="F7"/>
+      <x:c r="G7"/>
+      <x:c r="H7"/>
+      <x:c r="I7"/>
+      <x:c r="J7"/>
+      <x:c r="K7"/>
+      <x:c r="L7"/>
+      <x:c r="M7"/>
+      <x:c r="N7"/>
+      <x:c r="O7"/>
+      <x:c r="P7"/>
+      <x:c r="Q7"/>
+      <x:c r="R7"/>
+      <x:c r="S7"/>
+      <x:c r="T7"/>
+      <x:c r="U7"/>
+      <x:c r="V7"/>
+    </x:row>
+    <x:row r="8" ht="24" customHeight="1">
+      <x:c r="A8" s="84" t="str">
+        <x:v>EJEMPLOS: CARGOS</x:v>
+      </x:c>
+      <x:c r="B8" s="84"/>
+      <x:c r="C8" s="84"/>
+      <x:c r="D8" s="84"/>
+      <x:c r="E8" s="84"/>
+      <x:c r="F8" s="84"/>
+      <x:c r="G8" s="84"/>
+      <x:c r="H8" s="84"/>
+      <x:c r="I8" s="84"/>
+      <x:c r="J8" s="84"/>
+      <x:c r="K8" s="84"/>
+      <x:c r="L8" s="84"/>
+      <x:c r="M8" s="84"/>
+      <x:c r="N8" s="84"/>
+      <x:c r="O8" s="84"/>
+      <x:c r="P8" s="84"/>
+      <x:c r="Q8" s="84"/>
+      <x:c r="R8" s="84"/>
+      <x:c r="S8" s="84"/>
+      <x:c r="T8" s="84"/>
+      <x:c r="U8" s="84"/>
+      <x:c r="V8" s="84"/>
+    </x:row>
+    <x:row r="9" ht="42" customHeight="1">
+      <x:c r="A9" s="90" t="str">
+        <x:v>FOLIO O REFERENCIA DEL CARGO ANTERIOR</x:v>
+      </x:c>
+      <x:c r="B9" s="90" t="str">
+        <x:v>NÚMERO DE MEMBRESÍA</x:v>
+      </x:c>
+      <x:c r="C9" s="90" t="str">
+        <x:v>NOMBRE DEL CLUB</x:v>
+      </x:c>
+      <x:c r="D9" s="90" t="str">
+        <x:v>NÚMERO DE SOCIO</x:v>
+      </x:c>
+      <x:c r="E9" s="96" t="str">
+        <x:v>NOMBRE</x:v>
+      </x:c>
+      <x:c r="F9" s="96" t="str">
+        <x:v>APELLIDO PATERNO</x:v>
+      </x:c>
+      <x:c r="G9" s="96" t="str">
+        <x:v>APELLIDO MATERNO</x:v>
+      </x:c>
+      <x:c r="H9" s="96" t="str">
+        <x:v>TIPO DE MEMBRESÍA</x:v>
+      </x:c>
+      <x:c r="I9" s="90" t="str">
+        <x:v>CLAVE DEL CONCEPTO DE COBRO</x:v>
+      </x:c>
+      <x:c r="J9" s="90" t="str">
+        <x:v>NOMBRE DEL CONCEPTO DE COBRO</x:v>
+      </x:c>
+      <x:c r="K9" s="96" t="str">
+        <x:v>DESCRIPCIÓN DEL CARGO</x:v>
+      </x:c>
+      <x:c r="L9" s="96" t="str">
+        <x:v>IMPORTE ORIGINAL</x:v>
+      </x:c>
+      <x:c r="M9" s="96" t="str">
+        <x:v>SALDO PENDIENTE</x:v>
+      </x:c>
+      <x:c r="N9" s="96" t="str">
+        <x:v>FECHA DE EMISIÓN</x:v>
+      </x:c>
+      <x:c r="O9" s="96" t="str">
+        <x:v>FECHA DE VENCIMIENTO</x:v>
+      </x:c>
+      <x:c r="P9" s="96" t="str">
+        <x:v>AÑO DEL PERIODO</x:v>
+      </x:c>
+      <x:c r="Q9" s="96" t="str">
+        <x:v>MES DEL PERIODO</x:v>
+      </x:c>
+      <x:c r="R9" s="96" t="str">
+        <x:v>PERMITE ABONOS</x:v>
+      </x:c>
+      <x:c r="S9" s="90" t="str">
+        <x:v>ESTATUS</x:v>
+      </x:c>
+      <x:c r="T9" s="96" t="str">
+        <x:v>FECHA DE CANCELACIÓN</x:v>
+      </x:c>
+      <x:c r="U9" s="96" t="str">
+        <x:v>CORREO DE QUIEN CANCELÓ</x:v>
+      </x:c>
+      <x:c r="V9" s="96" t="str">
+        <x:v>MOTIVO DE CANCELACIÓN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="24" customHeight="1">
+      <x:c r="A10" s="101" t="str">
+        <x:v>CARGO-2026-1001</x:v>
+      </x:c>
+      <x:c r="B10" s="101" t="str">
+        <x:v>M-1001</x:v>
+      </x:c>
+      <x:c r="C10" s="101" t="str">
+        <x:v>PARQUE ESPAÑA</x:v>
+      </x:c>
+      <x:c r="D10" s="101" t="str">
+        <x:v>1001</x:v>
+      </x:c>
+      <x:c r="E10" s="101" t="str">
+        <x:v>Juan Carlos</x:v>
+      </x:c>
+      <x:c r="F10" s="101" t="str">
+        <x:v>Pérez</x:v>
+      </x:c>
+      <x:c r="G10" s="101" t="str">
+        <x:v>Hernández</x:v>
+      </x:c>
+      <x:c r="H10" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 1</x:v>
+      </x:c>
+      <x:c r="I10" s="101" t="str">
+        <x:v>EJ-001</x:v>
+      </x:c>
+      <x:c r="J10" s="101" t="str">
+        <x:v>CUOTA DE MANTENIMIENTO</x:v>
+      </x:c>
+      <x:c r="K10" s="101" t="str">
+        <x:v>Registro de ejemplo para el socio 1001.</x:v>
+      </x:c>
+      <x:c r="L10" s="103" t="n">
+        <x:v>2500</x:v>
+      </x:c>
+      <x:c r="M10" s="103" t="n">
+        <x:v>2500</x:v>
+      </x:c>
+      <x:c r="N10" s="102" t="n">
+        <x:v>46037</x:v>
+      </x:c>
+      <x:c r="O10" s="102" t="n">
+        <x:v>46037</x:v>
+      </x:c>
+      <x:c r="P10" s="101" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="Q10" s="101" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="R10" s="101" t="str">
+        <x:v>SÍ</x:v>
+      </x:c>
+      <x:c r="S10" s="101" t="str">
+        <x:v>ACTIVO</x:v>
+      </x:c>
+      <x:c r="T10" s="102" t="n">
+        <x:v>46037</x:v>
+      </x:c>
+      <x:c r="U10" s="101" t="str">
+        <x:v>juan.perez@example.com</x:v>
+      </x:c>
+      <x:c r="V10" s="101" t="str">
+        <x:v>Registro de ejemplo para el socio 1001.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="24" customHeight="1">
+      <x:c r="A11" s="101" t="str">
+        <x:v>CARGO-2026-1002</x:v>
+      </x:c>
+      <x:c r="B11" s="101" t="str">
+        <x:v>M-1002</x:v>
+      </x:c>
+      <x:c r="C11" s="101" t="str">
+        <x:v>PARQUE ESPAÑA</x:v>
+      </x:c>
+      <x:c r="D11" s="101" t="str">
+        <x:v>1002</x:v>
+      </x:c>
+      <x:c r="E11" s="101" t="str">
+        <x:v>María Fernanda</x:v>
+      </x:c>
+      <x:c r="F11" s="101" t="str">
+        <x:v>López</x:v>
+      </x:c>
+      <x:c r="G11" s="101" t="str">
+        <x:v>García</x:v>
+      </x:c>
+      <x:c r="H11" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 2</x:v>
+      </x:c>
+      <x:c r="I11" s="101" t="str">
+        <x:v>EJ-002</x:v>
+      </x:c>
+      <x:c r="J11" s="101" t="str">
+        <x:v>CUOTA DE CASILLERO</x:v>
+      </x:c>
+      <x:c r="K11" s="101" t="str">
+        <x:v>Registro de ejemplo para el socio 1002.</x:v>
+      </x:c>
+      <x:c r="L11" s="103" t="n">
+        <x:v>850</x:v>
+      </x:c>
+      <x:c r="M11" s="103" t="n">
+        <x:v>850</x:v>
+      </x:c>
+      <x:c r="N11" s="102" t="n">
+        <x:v>46044.291666666664</x:v>
+      </x:c>
+      <x:c r="O11" s="102" t="n">
+        <x:v>46044.291666666664</x:v>
+      </x:c>
+      <x:c r="P11" s="101" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="Q11" s="101" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="R11" s="101" t="str">
+        <x:v>SÍ</x:v>
+      </x:c>
+      <x:c r="S11" s="101" t="str">
+        <x:v>PENDIENTE</x:v>
+      </x:c>
+      <x:c r="T11" s="102" t="n">
+        <x:v>46044.291666666664</x:v>
+      </x:c>
+      <x:c r="U11" s="101" t="str">
+        <x:v>maria.lopez@example.com</x:v>
+      </x:c>
+      <x:c r="V11" s="101" t="str">
+        <x:v>Registro de ejemplo para el socio 1002.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="24" customHeight="1">
+      <x:c r="A12" s="101" t="str">
+        <x:v>CARGO-2026-1003</x:v>
+      </x:c>
+      <x:c r="B12" s="101" t="str">
+        <x:v>M-1003</x:v>
+      </x:c>
+      <x:c r="C12" s="101" t="str">
+        <x:v>PARQUE ESPAÑA</x:v>
+      </x:c>
+      <x:c r="D12" s="101" t="str">
+        <x:v>1003</x:v>
+      </x:c>
+      <x:c r="E12" s="101" t="str">
+        <x:v>Roberto</x:v>
+      </x:c>
+      <x:c r="F12" s="101" t="str">
+        <x:v>Sánchez</x:v>
+      </x:c>
+      <x:c r="G12" s="101" t="str">
+        <x:v>Morales</x:v>
+      </x:c>
+      <x:c r="H12" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 3</x:v>
+      </x:c>
+      <x:c r="I12" s="101" t="str">
+        <x:v>EJ-003</x:v>
+      </x:c>
+      <x:c r="J12" s="101" t="str">
+        <x:v>CLASE DE NATACIÓN</x:v>
+      </x:c>
+      <x:c r="K12" s="101" t="str">
+        <x:v>Registro de ejemplo para el socio 1003.</x:v>
+      </x:c>
+      <x:c r="L12" s="103" t="n">
+        <x:v>1200</x:v>
+      </x:c>
+      <x:c r="M12" s="103" t="n">
+        <x:v>1200</x:v>
+      </x:c>
+      <x:c r="N12" s="102" t="n">
+        <x:v>46051.333333333336</x:v>
+      </x:c>
+      <x:c r="O12" s="102" t="n">
+        <x:v>46051.333333333336</x:v>
+      </x:c>
+      <x:c r="P12" s="101" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="Q12" s="101" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="R12" s="101" t="str">
+        <x:v>SÍ</x:v>
+      </x:c>
+      <x:c r="S12" s="101" t="str">
+        <x:v>ACTIVO</x:v>
+      </x:c>
+      <x:c r="T12" s="102" t="n">
+        <x:v>46051.333333333336</x:v>
+      </x:c>
+      <x:c r="U12" s="101" t="str">
+        <x:v>roberto.sanchez@example.com</x:v>
+      </x:c>
+      <x:c r="V12" s="101" t="str">
+        <x:v>Registro de ejemplo para el socio 1003.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="24" customHeight="1">
+      <x:c r="A13"/>
+      <x:c r="B13"/>
+      <x:c r="C13"/>
+      <x:c r="D13"/>
+      <x:c r="E13"/>
+      <x:c r="F13"/>
+      <x:c r="G13"/>
+      <x:c r="H13"/>
+      <x:c r="I13"/>
+      <x:c r="J13"/>
+      <x:c r="K13"/>
+      <x:c r="L13"/>
+      <x:c r="M13"/>
+      <x:c r="N13"/>
+      <x:c r="O13"/>
+      <x:c r="P13"/>
+      <x:c r="Q13"/>
+      <x:c r="R13"/>
+      <x:c r="S13"/>
+      <x:c r="T13"/>
+    </x:row>
+    <x:row r="15" ht="24" customHeight="1">
+      <x:c r="A15" s="84" t="str">
+        <x:v>EJEMPLOS: PAGOS</x:v>
+      </x:c>
+      <x:c r="B15" s="84"/>
+      <x:c r="C15" s="84"/>
+      <x:c r="D15" s="84"/>
+      <x:c r="E15" s="84"/>
+      <x:c r="F15" s="84"/>
+      <x:c r="G15" s="84"/>
+      <x:c r="H15" s="84"/>
+      <x:c r="I15" s="84"/>
+      <x:c r="J15" s="84"/>
+      <x:c r="K15" s="84"/>
+      <x:c r="L15" s="84"/>
+      <x:c r="M15" s="84"/>
+      <x:c r="N15" s="84"/>
+      <x:c r="O15" s="84"/>
+      <x:c r="P15" s="84"/>
+      <x:c r="Q15" s="84"/>
+      <x:c r="R15" s="84"/>
+      <x:c r="S15" s="84"/>
+      <x:c r="T15" s="84"/>
+    </x:row>
+    <x:row r="16" ht="42" customHeight="1">
+      <x:c r="A16" s="90" t="str">
+        <x:v>FOLIO O REFERENCIA DEL PAGO ANTERIOR</x:v>
+      </x:c>
+      <x:c r="B16" s="96" t="str">
+        <x:v>FOLIO DEL COMPROBANTE</x:v>
+      </x:c>
+      <x:c r="C16" s="90" t="str">
+        <x:v>NÚMERO DE MEMBRESÍA</x:v>
+      </x:c>
+      <x:c r="D16" s="90" t="str">
+        <x:v>NOMBRE DEL CLUB</x:v>
+      </x:c>
+      <x:c r="E16" s="96" t="str">
+        <x:v>MÉTODO DE PAGO</x:v>
+      </x:c>
+      <x:c r="F16" s="96" t="str">
+        <x:v>IMPORTE PAGADO</x:v>
+      </x:c>
+      <x:c r="G16" s="96" t="str">
+        <x:v>SUBTOTAL</x:v>
+      </x:c>
+      <x:c r="H16" s="96" t="str">
+        <x:v>IVA</x:v>
+      </x:c>
+      <x:c r="I16" s="96" t="str">
+        <x:v>FECHA Y HORA DEL PAGO</x:v>
+      </x:c>
+      <x:c r="J16" s="96" t="str">
+        <x:v>REFERENCIA BANCARIA</x:v>
+      </x:c>
+      <x:c r="K16" s="96" t="str">
+        <x:v>NOMBRE DEL BANCO</x:v>
+      </x:c>
+      <x:c r="L16" s="96" t="str">
+        <x:v>NÚMERO DE CHEQUE</x:v>
+      </x:c>
+      <x:c r="M16" s="96" t="str">
+        <x:v>NOTAS</x:v>
+      </x:c>
+      <x:c r="N16" s="96" t="str">
+        <x:v>CORREO DE QUIEN RECIBIÓ</x:v>
+      </x:c>
+      <x:c r="O16" s="90" t="str">
+        <x:v>ESTATUS</x:v>
+      </x:c>
+      <x:c r="P16" s="96" t="str">
+        <x:v>NOMBRE DEL ARCHIVO DEL COMPROBANTE</x:v>
+      </x:c>
+      <x:c r="Q16" s="96" t="str">
+        <x:v>REFERENCIA DE LA OPERACIÓN AGRUPADA</x:v>
+      </x:c>
+      <x:c r="R16" s="96" t="str">
+        <x:v>FECHA DE CANCELACIÓN</x:v>
+      </x:c>
+      <x:c r="S16" s="96" t="str">
+        <x:v>CORREO DE QUIEN CANCELÓ</x:v>
+      </x:c>
+      <x:c r="T16" s="96" t="str">
+        <x:v>MOTIVO DE CANCELACIÓN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="24" customHeight="1">
+      <x:c r="A17" s="101" t="str">
+        <x:v>PAGO-2026-1001</x:v>
+      </x:c>
+      <x:c r="B17" s="101" t="str">
+        <x:v>REF-2026-001</x:v>
+      </x:c>
+      <x:c r="C17" s="101" t="str">
+        <x:v>M-1001</x:v>
+      </x:c>
+      <x:c r="D17" s="101" t="str">
+        <x:v>PARQUE ESPAÑA</x:v>
+      </x:c>
+      <x:c r="E17" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 1</x:v>
+      </x:c>
+      <x:c r="F17" s="103" t="n">
+        <x:v>2500</x:v>
+      </x:c>
+      <x:c r="G17" s="103" t="n">
+        <x:v>2500</x:v>
+      </x:c>
+      <x:c r="H17" s="103" t="n">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="I17" s="104" t="n">
+        <x:v>46037.625</x:v>
+      </x:c>
+      <x:c r="J17" s="101" t="str">
+        <x:v>REF-2026-001</x:v>
+      </x:c>
+      <x:c r="K17" s="101" t="str">
+        <x:v>BBVA</x:v>
+      </x:c>
+      <x:c r="L17" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 1</x:v>
+      </x:c>
+      <x:c r="M17" s="101" t="str">
+        <x:v>Registro de ejemplo para el socio 1001.</x:v>
+      </x:c>
+      <x:c r="N17" s="101" t="str">
+        <x:v>juan.perez@example.com</x:v>
+      </x:c>
+      <x:c r="O17" s="101" t="str">
+        <x:v>ACTIVO</x:v>
+      </x:c>
+      <x:c r="P17" s="101" t="str">
+        <x:v>documentos/socio-1001.pdf</x:v>
+      </x:c>
+      <x:c r="Q17" s="101" t="str">
+        <x:v>REF-2026-001</x:v>
+      </x:c>
+      <x:c r="R17" s="102" t="n">
+        <x:v>46037</x:v>
+      </x:c>
+      <x:c r="S17" s="101" t="str">
+        <x:v>juan.perez@example.com</x:v>
+      </x:c>
+      <x:c r="T17" s="101" t="str">
+        <x:v>Registro de ejemplo para el socio 1001.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="24" customHeight="1">
+      <x:c r="A18" s="101" t="str">
+        <x:v>PAGO-2026-1002</x:v>
+      </x:c>
+      <x:c r="B18" s="101" t="str">
+        <x:v>REF-2026-002</x:v>
+      </x:c>
+      <x:c r="C18" s="101" t="str">
+        <x:v>M-1002</x:v>
+      </x:c>
+      <x:c r="D18" s="101" t="str">
+        <x:v>PARQUE ESPAÑA</x:v>
+      </x:c>
+      <x:c r="E18" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 2</x:v>
+      </x:c>
+      <x:c r="F18" s="103" t="n">
+        <x:v>850</x:v>
+      </x:c>
+      <x:c r="G18" s="103" t="n">
+        <x:v>850</x:v>
+      </x:c>
+      <x:c r="H18" s="103" t="n">
+        <x:v>136</x:v>
+      </x:c>
+      <x:c r="I18" s="104" t="n">
+        <x:v>46044.666666666664</x:v>
+      </x:c>
+      <x:c r="J18" s="101" t="str">
+        <x:v>REF-2026-002</x:v>
+      </x:c>
+      <x:c r="K18" s="101" t="str">
+        <x:v>BANORTE</x:v>
+      </x:c>
+      <x:c r="L18" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 2</x:v>
+      </x:c>
+      <x:c r="M18" s="101" t="str">
+        <x:v>Registro de ejemplo para el socio 1002.</x:v>
+      </x:c>
+      <x:c r="N18" s="101" t="str">
+        <x:v>maria.lopez@example.com</x:v>
+      </x:c>
+      <x:c r="O18" s="101" t="str">
+        <x:v>PENDIENTE</x:v>
+      </x:c>
+      <x:c r="P18" s="101" t="str">
+        <x:v>documentos/socio-1002.pdf</x:v>
+      </x:c>
+      <x:c r="Q18" s="101" t="str">
+        <x:v>REF-2026-002</x:v>
+      </x:c>
+      <x:c r="R18" s="102" t="n">
+        <x:v>46044.291666666664</x:v>
+      </x:c>
+      <x:c r="S18" s="101" t="str">
+        <x:v>maria.lopez@example.com</x:v>
+      </x:c>
+      <x:c r="T18" s="101" t="str">
+        <x:v>Registro de ejemplo para el socio 1002.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="24" customHeight="1">
+      <x:c r="A19" s="101" t="str">
+        <x:v>PAGO-2026-1003</x:v>
+      </x:c>
+      <x:c r="B19" s="101" t="str">
+        <x:v>REF-2026-003</x:v>
+      </x:c>
+      <x:c r="C19" s="101" t="str">
+        <x:v>M-1003</x:v>
+      </x:c>
+      <x:c r="D19" s="101" t="str">
+        <x:v>PARQUE ESPAÑA</x:v>
+      </x:c>
+      <x:c r="E19" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 3</x:v>
+      </x:c>
+      <x:c r="F19" s="103" t="n">
+        <x:v>1200</x:v>
+      </x:c>
+      <x:c r="G19" s="103" t="n">
+        <x:v>1200</x:v>
+      </x:c>
+      <x:c r="H19" s="103" t="n">
+        <x:v>192</x:v>
+      </x:c>
+      <x:c r="I19" s="104" t="n">
+        <x:v>46051.708333333336</x:v>
+      </x:c>
+      <x:c r="J19" s="101" t="str">
+        <x:v>REF-2026-003</x:v>
+      </x:c>
+      <x:c r="K19" s="101" t="str">
+        <x:v>SANTANDER</x:v>
+      </x:c>
+      <x:c r="L19" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 3</x:v>
+      </x:c>
+      <x:c r="M19" s="101" t="str">
+        <x:v>Registro de ejemplo para el socio 1003.</x:v>
+      </x:c>
+      <x:c r="N19" s="101" t="str">
+        <x:v>roberto.sanchez@example.com</x:v>
+      </x:c>
+      <x:c r="O19" s="101" t="str">
+        <x:v>ACTIVO</x:v>
+      </x:c>
+      <x:c r="P19" s="101" t="str">
+        <x:v>documentos/socio-1003.pdf</x:v>
+      </x:c>
+      <x:c r="Q19" s="101" t="str">
+        <x:v>REF-2026-003</x:v>
+      </x:c>
+      <x:c r="R19" s="102" t="n">
+        <x:v>46051.333333333336</x:v>
+      </x:c>
+      <x:c r="S19" s="101" t="str">
+        <x:v>roberto.sanchez@example.com</x:v>
+      </x:c>
+      <x:c r="T19" s="101" t="str">
+        <x:v>Registro de ejemplo para el socio 1003.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="24" customHeight="1">
+      <x:c r="A21"/>
+      <x:c r="B21"/>
+      <x:c r="C21"/>
+      <x:c r="D21"/>
+    </x:row>
+    <x:row r="22" ht="24" customHeight="1">
+      <x:c r="A22" s="84" t="str">
+        <x:v>EJEMPLOS: APLICACIONES DE PAGOS</x:v>
+      </x:c>
+      <x:c r="B22" s="84"/>
+      <x:c r="C22" s="84"/>
+      <x:c r="D22" s="84"/>
+      <x:c r="E22" s="84"/>
+      <x:c r="F22" s="84"/>
+      <x:c r="G22" s="84"/>
+      <x:c r="H22" s="84"/>
+      <x:c r="I22" s="84"/>
+      <x:c r="J22" s="84"/>
+      <x:c r="K22" s="84"/>
+      <x:c r="L22" s="84"/>
+    </x:row>
+    <x:row r="23" ht="42" customHeight="1">
+      <x:c r="A23" s="90" t="str">
+        <x:v>FOLIO O REFERENCIA DEL PAGO ANTERIOR</x:v>
+      </x:c>
+      <x:c r="B23" s="96" t="str">
+        <x:v>FOLIO DEL COMPROBANTE</x:v>
+      </x:c>
+      <x:c r="C23" s="90" t="str">
+        <x:v>FOLIO O REFERENCIA DEL CARGO ANTERIOR</x:v>
+      </x:c>
+      <x:c r="D23" s="90" t="str">
+        <x:v>NÚMERO DE MEMBRESÍA</x:v>
+      </x:c>
+      <x:c r="E23" s="90" t="str">
+        <x:v>CLAVE DEL CONCEPTO DE COBRO</x:v>
+      </x:c>
+      <x:c r="F23" s="90" t="str">
+        <x:v>NOMBRE DEL CONCEPTO DE COBRO</x:v>
+      </x:c>
+      <x:c r="G23" s="96" t="str">
+        <x:v>DESCRIPCIÓN DEL CARGO</x:v>
+      </x:c>
+      <x:c r="H23" s="96" t="str">
+        <x:v>FECHA DE EMISIÓN DEL CARGO</x:v>
+      </x:c>
+      <x:c r="I23" s="96" t="str">
+        <x:v>IMPORTE APLICADO</x:v>
+      </x:c>
+      <x:c r="J23" s="96" t="str">
+        <x:v>SUBTOTAL APLICADO</x:v>
+      </x:c>
+      <x:c r="K23" s="96" t="str">
+        <x:v>IVA APLICADO</x:v>
+      </x:c>
+      <x:c r="L23" s="96" t="str">
+        <x:v>DESCUENTO APLICADO</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="24" customHeight="1">
+      <x:c r="A24" s="101" t="str">
+        <x:v>PAGO-2026-1001</x:v>
+      </x:c>
+      <x:c r="B24" s="101" t="str">
+        <x:v>REF-2026-001</x:v>
+      </x:c>
+      <x:c r="C24" s="101" t="str">
+        <x:v>CARGO-2026-1001</x:v>
+      </x:c>
+      <x:c r="D24" s="101" t="str">
+        <x:v>M-1001</x:v>
+      </x:c>
+      <x:c r="E24" s="101" t="str">
+        <x:v>EJ-001</x:v>
+      </x:c>
+      <x:c r="F24" s="101" t="str">
+        <x:v>CUOTA DE MANTENIMIENTO</x:v>
+      </x:c>
+      <x:c r="G24" s="101" t="str">
+        <x:v>Registro de ejemplo para el socio 1001.</x:v>
+      </x:c>
+      <x:c r="H24" s="102" t="n">
+        <x:v>46037</x:v>
+      </x:c>
+      <x:c r="I24" s="103" t="n">
+        <x:v>2500</x:v>
+      </x:c>
+      <x:c r="J24" s="103" t="n">
+        <x:v>2500</x:v>
+      </x:c>
+      <x:c r="K24" s="103" t="n">
+        <x:v>400</x:v>
+      </x:c>
+      <x:c r="L24" s="101" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="24" customHeight="1">
+      <x:c r="A25" s="101" t="str">
+        <x:v>PAGO-2026-1002</x:v>
+      </x:c>
+      <x:c r="B25" s="101" t="str">
+        <x:v>REF-2026-002</x:v>
+      </x:c>
+      <x:c r="C25" s="101" t="str">
+        <x:v>CARGO-2026-1002</x:v>
+      </x:c>
+      <x:c r="D25" s="101" t="str">
+        <x:v>M-1002</x:v>
+      </x:c>
+      <x:c r="E25" s="101" t="str">
+        <x:v>EJ-002</x:v>
+      </x:c>
+      <x:c r="F25" s="101" t="str">
+        <x:v>CUOTA DE CASILLERO</x:v>
+      </x:c>
+      <x:c r="G25" s="101" t="str">
+        <x:v>Registro de ejemplo para el socio 1002.</x:v>
+      </x:c>
+      <x:c r="H25" s="102" t="n">
+        <x:v>46044.291666666664</x:v>
+      </x:c>
+      <x:c r="I25" s="103" t="n">
+        <x:v>850</x:v>
+      </x:c>
+      <x:c r="J25" s="103" t="n">
+        <x:v>850</x:v>
+      </x:c>
+      <x:c r="K25" s="103" t="n">
+        <x:v>136</x:v>
+      </x:c>
+      <x:c r="L25" s="101" t="n">
+        <x:v>85</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="24" customHeight="1">
+      <x:c r="A26" s="101" t="str">
+        <x:v>PAGO-2026-1003</x:v>
+      </x:c>
+      <x:c r="B26" s="101" t="str">
+        <x:v>REF-2026-003</x:v>
+      </x:c>
+      <x:c r="C26" s="101" t="str">
+        <x:v>CARGO-2026-1003</x:v>
+      </x:c>
+      <x:c r="D26" s="101" t="str">
+        <x:v>M-1003</x:v>
+      </x:c>
+      <x:c r="E26" s="101" t="str">
+        <x:v>EJ-003</x:v>
+      </x:c>
+      <x:c r="F26" s="101" t="str">
+        <x:v>CLASE DE NATACIÓN</x:v>
+      </x:c>
+      <x:c r="G26" s="101" t="str">
+        <x:v>Registro de ejemplo para el socio 1003.</x:v>
+      </x:c>
+      <x:c r="H26" s="102" t="n">
+        <x:v>46051.333333333336</x:v>
+      </x:c>
+      <x:c r="I26" s="103" t="n">
+        <x:v>1200</x:v>
+      </x:c>
+      <x:c r="J26" s="103" t="n">
+        <x:v>1200</x:v>
+      </x:c>
+      <x:c r="K26" s="103" t="n">
+        <x:v>192</x:v>
+      </x:c>
+      <x:c r="L26" s="101" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="42" customHeight="1">
+      <x:c r="A27"/>
+      <x:c r="B27"/>
+      <x:c r="C27"/>
+      <x:c r="D27"/>
+      <x:c r="E27"/>
+      <x:c r="F27"/>
+      <x:c r="G27"/>
+      <x:c r="H27"/>
+    </x:row>
+    <x:row r="28" ht="24" customHeight="1">
+      <x:c r="A28"/>
+      <x:c r="B28"/>
+      <x:c r="C28"/>
+      <x:c r="D28"/>
+      <x:c r="E28"/>
+      <x:c r="F28"/>
+      <x:c r="G28"/>
+      <x:c r="H28"/>
+    </x:row>
+    <x:row r="29" ht="24" customHeight="1">
+      <x:c r="A29" s="84" t="str">
+        <x:v>EJEMPLOS: SALDOS A FAVOR</x:v>
+      </x:c>
+      <x:c r="B29" s="84"/>
+      <x:c r="C29" s="84"/>
+      <x:c r="D29" s="84"/>
+    </x:row>
+    <x:row r="30" ht="42" customHeight="1">
+      <x:c r="A30" s="90" t="str">
+        <x:v>NÚMERO DE MEMBRESÍA</x:v>
+      </x:c>
+      <x:c r="B30" s="90" t="str">
+        <x:v>NOMBRE DEL CLUB</x:v>
+      </x:c>
+      <x:c r="C30" s="96" t="str">
+        <x:v>IMPORTE DEL SALDO A FAVOR</x:v>
+      </x:c>
+      <x:c r="D30" s="96" t="str">
+        <x:v>FECHA DE CORTE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="24" customHeight="1">
+      <x:c r="A31" s="101" t="str">
+        <x:v>M-1001</x:v>
+      </x:c>
+      <x:c r="B31" s="101" t="str">
+        <x:v>PARQUE ESPAÑA</x:v>
+      </x:c>
+      <x:c r="C31" s="103" t="n">
+        <x:v>2500</x:v>
+      </x:c>
+      <x:c r="D31" s="102" t="n">
+        <x:v>46037</x:v>
+      </x:c>
+      <x:c r="E31"/>
+    </x:row>
+    <x:row r="32" ht="24" customHeight="1">
+      <x:c r="A32" s="101" t="str">
+        <x:v>M-1002</x:v>
+      </x:c>
+      <x:c r="B32" s="101" t="str">
+        <x:v>PARQUE ESPAÑA</x:v>
+      </x:c>
+      <x:c r="C32" s="103" t="n">
+        <x:v>850</x:v>
+      </x:c>
+      <x:c r="D32" s="102" t="n">
+        <x:v>46044.291666666664</x:v>
+      </x:c>
+      <x:c r="E32"/>
+    </x:row>
+    <x:row r="33" ht="24" customHeight="1">
+      <x:c r="A33" s="101" t="str">
+        <x:v>M-1003</x:v>
+      </x:c>
+      <x:c r="B33" s="101" t="str">
+        <x:v>PARQUE ESPAÑA</x:v>
+      </x:c>
+      <x:c r="C33" s="103" t="n">
+        <x:v>1200</x:v>
+      </x:c>
+      <x:c r="D33" s="102" t="n">
+        <x:v>46051.333333333336</x:v>
+      </x:c>
+      <x:c r="E33"/>
+    </x:row>
+    <x:row r="36" ht="24" customHeight="1">
+      <x:c r="A36" s="84" t="str">
+        <x:v>EJEMPLOS: MOVIMIENTOS DE SALDO</x:v>
+      </x:c>
+      <x:c r="B36" s="84"/>
+      <x:c r="C36" s="84"/>
+      <x:c r="D36" s="84"/>
+      <x:c r="E36" s="84"/>
+      <x:c r="F36" s="84"/>
+      <x:c r="G36" s="84"/>
+      <x:c r="H36" s="84"/>
+      <x:c r="I36"/>
+      <x:c r="J36"/>
+      <x:c r="K36"/>
+      <x:c r="L36"/>
+      <x:c r="M36"/>
+    </x:row>
+    <x:row r="37" ht="42" customHeight="1">
+      <x:c r="A37" s="90" t="str">
+        <x:v>NÚMERO DE MEMBRESÍA</x:v>
+      </x:c>
+      <x:c r="B37" s="90" t="str">
+        <x:v>NOMBRE DEL CLUB</x:v>
+      </x:c>
+      <x:c r="C37" s="96" t="str">
+        <x:v>FECHA Y HORA DEL MOVIMIENTO</x:v>
+      </x:c>
+      <x:c r="D37" s="96" t="str">
+        <x:v>IMPORTE DEL MOVIMIENTO</x:v>
+      </x:c>
+      <x:c r="E37" s="96" t="str">
+        <x:v>CONCEPTO DEL MOVIMIENTO</x:v>
+      </x:c>
+      <x:c r="F37" s="90" t="str">
+        <x:v>FOLIO O REFERENCIA DEL CARGO ANTERIOR</x:v>
+      </x:c>
+      <x:c r="G37" s="90" t="str">
+        <x:v>FOLIO O REFERENCIA DEL PAGO ANTERIOR</x:v>
+      </x:c>
+      <x:c r="H37" s="96" t="str">
+        <x:v>NOTAS</x:v>
+      </x:c>
+      <x:c r="I37"/>
+      <x:c r="J37"/>
+      <x:c r="K37"/>
+      <x:c r="L37"/>
+      <x:c r="M37"/>
+    </x:row>
+    <x:row r="38" ht="24" customHeight="1">
+      <x:c r="A38" s="101" t="str">
+        <x:v>M-1001</x:v>
+      </x:c>
+      <x:c r="B38" s="101" t="str">
+        <x:v>PARQUE ESPAÑA</x:v>
+      </x:c>
+      <x:c r="C38" s="104" t="n">
+        <x:v>46037.625</x:v>
+      </x:c>
+      <x:c r="D38" s="103" t="n">
+        <x:v>2500</x:v>
+      </x:c>
+      <x:c r="E38" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 1</x:v>
+      </x:c>
+      <x:c r="F38" s="101" t="str">
+        <x:v>CARGO-2026-1001</x:v>
+      </x:c>
+      <x:c r="G38" s="101" t="str">
+        <x:v>PAGO-2026-1001</x:v>
+      </x:c>
+      <x:c r="H38" s="101" t="str">
+        <x:v>Registro de ejemplo para el socio 1001.</x:v>
+      </x:c>
+      <x:c r="I38"/>
+      <x:c r="J38"/>
+      <x:c r="K38"/>
+      <x:c r="L38"/>
+      <x:c r="M38"/>
+    </x:row>
+    <x:row r="39" ht="24" customHeight="1">
+      <x:c r="A39" s="101" t="str">
+        <x:v>M-1002</x:v>
+      </x:c>
+      <x:c r="B39" s="101" t="str">
+        <x:v>PARQUE ESPAÑA</x:v>
+      </x:c>
+      <x:c r="C39" s="104" t="n">
+        <x:v>46044.666666666664</x:v>
+      </x:c>
+      <x:c r="D39" s="103" t="n">
+        <x:v>850</x:v>
+      </x:c>
+      <x:c r="E39" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 2</x:v>
+      </x:c>
+      <x:c r="F39" s="101" t="str">
+        <x:v>CARGO-2026-1002</x:v>
+      </x:c>
+      <x:c r="G39" s="101" t="str">
+        <x:v>PAGO-2026-1002</x:v>
+      </x:c>
+      <x:c r="H39" s="101" t="str">
+        <x:v>Registro de ejemplo para el socio 1002.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="24" customHeight="1">
+      <x:c r="A40" s="101" t="str">
+        <x:v>M-1003</x:v>
+      </x:c>
+      <x:c r="B40" s="101" t="str">
+        <x:v>PARQUE ESPAÑA</x:v>
+      </x:c>
+      <x:c r="C40" s="104" t="n">
+        <x:v>46051.708333333336</x:v>
+      </x:c>
+      <x:c r="D40" s="103" t="n">
+        <x:v>1200</x:v>
+      </x:c>
+      <x:c r="E40" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 3</x:v>
+      </x:c>
+      <x:c r="F40" s="101" t="str">
+        <x:v>CARGO-2026-1003</x:v>
+      </x:c>
+      <x:c r="G40" s="101" t="str">
+        <x:v>PAGO-2026-1003</x:v>
+      </x:c>
+      <x:c r="H40" s="101" t="str">
+        <x:v>Registro de ejemplo para el socio 1003.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="24" customHeight="1">
+      <x:c r="A41"/>
+      <x:c r="B41"/>
+      <x:c r="C41"/>
+      <x:c r="D41"/>
+      <x:c r="E41"/>
+      <x:c r="F41"/>
+      <x:c r="G41"/>
+      <x:c r="H41"/>
+    </x:row>
+    <x:row r="42" ht="42" customHeight="1">
+      <x:c r="A42"/>
+      <x:c r="B42"/>
+      <x:c r="C42"/>
+      <x:c r="D42"/>
+      <x:c r="E42"/>
+      <x:c r="F42"/>
+      <x:c r="G42"/>
+      <x:c r="H42"/>
+    </x:row>
+    <x:row r="43" ht="24" customHeight="1">
+      <x:c r="A43" s="84" t="str">
+        <x:v>EJEMPLOS: NOTAS DE COBRANZA</x:v>
+      </x:c>
+      <x:c r="B43" s="84"/>
+      <x:c r="C43" s="84"/>
+      <x:c r="D43" s="84"/>
+      <x:c r="E43" s="84"/>
+      <x:c r="F43"/>
+      <x:c r="G43"/>
+      <x:c r="H43"/>
+    </x:row>
+    <x:row r="44" ht="42" customHeight="1">
+      <x:c r="A44" s="90" t="str">
+        <x:v>NÚMERO DE MEMBRESÍA</x:v>
+      </x:c>
+      <x:c r="B44" s="90" t="str">
+        <x:v>NOMBRE DEL CLUB</x:v>
+      </x:c>
+      <x:c r="C44" s="96" t="str">
+        <x:v>FECHA Y HORA DE LA NOTA</x:v>
+      </x:c>
+      <x:c r="D44" s="96" t="str">
+        <x:v>CORREO DE QUIEN REGISTRÓ LA NOTA</x:v>
+      </x:c>
+      <x:c r="E44" s="96" t="str">
+        <x:v>NOTA DE COBRANZA</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="24" customHeight="1">
+      <x:c r="A45" s="101" t="str">
+        <x:v>M-1001</x:v>
+      </x:c>
+      <x:c r="B45" s="101" t="str">
+        <x:v>PARQUE ESPAÑA</x:v>
+      </x:c>
+      <x:c r="C45" s="104" t="n">
+        <x:v>46037.625</x:v>
+      </x:c>
+      <x:c r="D45" s="101" t="str">
+        <x:v>juan.perez@example.com</x:v>
+      </x:c>
+      <x:c r="E45" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="24" customHeight="1">
+      <x:c r="A46" s="101" t="str">
+        <x:v>M-1002</x:v>
+      </x:c>
+      <x:c r="B46" s="101" t="str">
+        <x:v>PARQUE ESPAÑA</x:v>
+      </x:c>
+      <x:c r="C46" s="104" t="n">
+        <x:v>46044.666666666664</x:v>
+      </x:c>
+      <x:c r="D46" s="101" t="str">
+        <x:v>maria.lopez@example.com</x:v>
+      </x:c>
+      <x:c r="E46" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 2</x:v>
+      </x:c>
+      <x:c r="F46"/>
+      <x:c r="G46"/>
+      <x:c r="H46"/>
+      <x:c r="I46"/>
+      <x:c r="J46"/>
+      <x:c r="K46"/>
+      <x:c r="L46"/>
+      <x:c r="M46"/>
+      <x:c r="N46"/>
+    </x:row>
+    <x:row r="47" ht="24" customHeight="1">
+      <x:c r="A47" s="101" t="str">
+        <x:v>M-1003</x:v>
+      </x:c>
+      <x:c r="B47" s="101" t="str">
+        <x:v>PARQUE ESPAÑA</x:v>
+      </x:c>
+      <x:c r="C47" s="104" t="n">
+        <x:v>46051.708333333336</x:v>
+      </x:c>
+      <x:c r="D47" s="101" t="str">
+        <x:v>roberto.sanchez@example.com</x:v>
+      </x:c>
+      <x:c r="E47" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 3</x:v>
+      </x:c>
+      <x:c r="F47"/>
+      <x:c r="G47"/>
+      <x:c r="H47"/>
+      <x:c r="I47"/>
+      <x:c r="J47"/>
+      <x:c r="K47"/>
+      <x:c r="L47"/>
+      <x:c r="M47"/>
+      <x:c r="N47"/>
+    </x:row>
+    <x:row r="48" ht="24" customHeight="1">
+      <x:c r="A48"/>
+      <x:c r="B48"/>
+      <x:c r="C48"/>
+      <x:c r="D48"/>
+      <x:c r="E48"/>
+      <x:c r="F48"/>
+      <x:c r="G48"/>
+      <x:c r="H48"/>
+      <x:c r="I48"/>
+      <x:c r="J48"/>
+      <x:c r="K48"/>
+      <x:c r="L48"/>
+      <x:c r="M48"/>
+      <x:c r="N48"/>
+    </x:row>
+    <x:row r="50" ht="24" customHeight="1">
+      <x:c r="A50" s="84" t="str">
+        <x:v>EJEMPLOS: OPERACIONES SPEI</x:v>
+      </x:c>
+      <x:c r="B50" s="84"/>
+      <x:c r="C50" s="84"/>
+      <x:c r="D50" s="84"/>
+      <x:c r="E50" s="84"/>
+      <x:c r="F50" s="84"/>
+      <x:c r="G50" s="84"/>
+      <x:c r="H50" s="84"/>
+      <x:c r="I50" s="84"/>
+      <x:c r="J50" s="84"/>
+      <x:c r="K50" s="84"/>
+      <x:c r="L50" s="84"/>
+      <x:c r="M50" s="84"/>
+    </x:row>
+    <x:row r="51" ht="42" customHeight="1">
+      <x:c r="A51" s="90" t="str">
+        <x:v>FOLIO O REFERENCIA DE LA OPERACIÓN ANTERIOR</x:v>
+      </x:c>
+      <x:c r="B51" s="90" t="str">
+        <x:v>NÚMERO DE MEMBRESÍA</x:v>
+      </x:c>
+      <x:c r="C51" s="90" t="str">
+        <x:v>NOMBRE DEL CLUB</x:v>
+      </x:c>
+      <x:c r="D51" s="96" t="str">
+        <x:v>MÉTODO DE PAGO</x:v>
+      </x:c>
+      <x:c r="E51" s="96" t="str">
+        <x:v>FOLIO DE LA ORDEN EN EL PROVEEDOR</x:v>
+      </x:c>
+      <x:c r="F51" s="96" t="str">
+        <x:v>FOLIO DEL CARGO EN EL PROVEEDOR</x:v>
+      </x:c>
+      <x:c r="G51" s="96" t="str">
+        <x:v>CLABE</x:v>
+      </x:c>
+      <x:c r="H51" s="96" t="str">
+        <x:v>NOMBRE DEL BANCO</x:v>
+      </x:c>
+      <x:c r="I51" s="96" t="str">
+        <x:v>IMPORTE</x:v>
+      </x:c>
+      <x:c r="J51" s="96" t="str">
+        <x:v>FECHA Y HORA DE VENCIMIENTO</x:v>
+      </x:c>
+      <x:c r="K51" s="90" t="str">
+        <x:v>ESTATUS</x:v>
+      </x:c>
+      <x:c r="L51" s="90" t="str">
+        <x:v>FOLIO O REFERENCIA DEL PAGO ANTERIOR</x:v>
+      </x:c>
+      <x:c r="M51" s="96" t="str">
+        <x:v>NOTAS</x:v>
+      </x:c>
+      <x:c r="N51"/>
+    </x:row>
+    <x:row r="52" ht="24" customHeight="1">
+      <x:c r="A52" s="101" t="str">
+        <x:v>REF-2026-001</x:v>
+      </x:c>
+      <x:c r="B52" s="101" t="str">
+        <x:v>M-1001</x:v>
+      </x:c>
+      <x:c r="C52" s="101" t="str">
+        <x:v>PARQUE ESPAÑA</x:v>
+      </x:c>
+      <x:c r="D52" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 1</x:v>
+      </x:c>
+      <x:c r="E52" s="101" t="str">
+        <x:v>REF-2026-001</x:v>
+      </x:c>
+      <x:c r="F52" s="101" t="str">
+        <x:v>REF-2026-001</x:v>
+      </x:c>
+      <x:c r="G52" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 1</x:v>
+      </x:c>
+      <x:c r="H52" s="101" t="str">
+        <x:v>BBVA</x:v>
+      </x:c>
+      <x:c r="I52" s="103" t="n">
+        <x:v>2500</x:v>
+      </x:c>
+      <x:c r="J52" s="104" t="n">
+        <x:v>46037.625</x:v>
+      </x:c>
+      <x:c r="K52" s="101" t="str">
+        <x:v>ACTIVO</x:v>
+      </x:c>
+      <x:c r="L52" s="101" t="str">
+        <x:v>PAGO-2026-1001</x:v>
+      </x:c>
+      <x:c r="M52" s="101" t="str">
+        <x:v>Registro de ejemplo para el socio 1001.</x:v>
+      </x:c>
+      <x:c r="N52"/>
+    </x:row>
+    <x:row r="53" ht="24" customHeight="1">
+      <x:c r="A53" s="101" t="str">
+        <x:v>REF-2026-002</x:v>
+      </x:c>
+      <x:c r="B53" s="101" t="str">
+        <x:v>M-1002</x:v>
+      </x:c>
+      <x:c r="C53" s="101" t="str">
+        <x:v>PARQUE ESPAÑA</x:v>
+      </x:c>
+      <x:c r="D53" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 2</x:v>
+      </x:c>
+      <x:c r="E53" s="101" t="str">
+        <x:v>REF-2026-002</x:v>
+      </x:c>
+      <x:c r="F53" s="101" t="str">
+        <x:v>REF-2026-002</x:v>
+      </x:c>
+      <x:c r="G53" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 2</x:v>
+      </x:c>
+      <x:c r="H53" s="101" t="str">
+        <x:v>BANORTE</x:v>
+      </x:c>
+      <x:c r="I53" s="103" t="n">
+        <x:v>850</x:v>
+      </x:c>
+      <x:c r="J53" s="104" t="n">
+        <x:v>46044.666666666664</x:v>
+      </x:c>
+      <x:c r="K53" s="101" t="str">
+        <x:v>PENDIENTE</x:v>
+      </x:c>
+      <x:c r="L53" s="101" t="str">
+        <x:v>PAGO-2026-1002</x:v>
+      </x:c>
+      <x:c r="M53" s="101" t="str">
+        <x:v>Registro de ejemplo para el socio 1002.</x:v>
+      </x:c>
+      <x:c r="N53"/>
+    </x:row>
+    <x:row r="54" ht="24" customHeight="1">
+      <x:c r="A54" s="101" t="str">
+        <x:v>REF-2026-003</x:v>
+      </x:c>
+      <x:c r="B54" s="101" t="str">
+        <x:v>M-1003</x:v>
+      </x:c>
+      <x:c r="C54" s="101" t="str">
+        <x:v>PARQUE ESPAÑA</x:v>
+      </x:c>
+      <x:c r="D54" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 3</x:v>
+      </x:c>
+      <x:c r="E54" s="101" t="str">
+        <x:v>REF-2026-003</x:v>
+      </x:c>
+      <x:c r="F54" s="101" t="str">
+        <x:v>REF-2026-003</x:v>
+      </x:c>
+      <x:c r="G54" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 3</x:v>
+      </x:c>
+      <x:c r="H54" s="101" t="str">
+        <x:v>SANTANDER</x:v>
+      </x:c>
+      <x:c r="I54" s="103" t="n">
+        <x:v>1200</x:v>
+      </x:c>
+      <x:c r="J54" s="104" t="n">
+        <x:v>46051.708333333336</x:v>
+      </x:c>
+      <x:c r="K54" s="101" t="str">
+        <x:v>ACTIVO</x:v>
+      </x:c>
+      <x:c r="L54" s="101" t="str">
+        <x:v>PAGO-2026-1003</x:v>
+      </x:c>
+      <x:c r="M54" s="101" t="str">
+        <x:v>Registro de ejemplo para el socio 1003.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="24" customHeight="1">
+      <x:c r="A56"/>
+      <x:c r="B56"/>
+      <x:c r="C56"/>
+      <x:c r="D56"/>
+      <x:c r="E56"/>
+      <x:c r="F56"/>
+      <x:c r="G56"/>
+    </x:row>
+    <x:row r="57" ht="24" customHeight="1">
+      <x:c r="A57" s="84" t="str">
+        <x:v>EJEMPLOS: APLICACIONES SPEI</x:v>
+      </x:c>
+      <x:c r="B57" s="84"/>
+      <x:c r="C57" s="84"/>
+      <x:c r="D57" s="84"/>
+      <x:c r="E57" s="84"/>
+      <x:c r="F57" s="84"/>
+      <x:c r="G57" s="84"/>
+      <x:c r="H57" s="84"/>
+    </x:row>
+    <x:row r="58" ht="42" customHeight="1">
+      <x:c r="A58" s="90" t="str">
+        <x:v>FOLIO O REFERENCIA DE LA OPERACIÓN ANTERIOR</x:v>
+      </x:c>
+      <x:c r="B58" s="90" t="str">
+        <x:v>NÚMERO DE MEMBRESÍA</x:v>
+      </x:c>
+      <x:c r="C58" s="90" t="str">
+        <x:v>FOLIO O REFERENCIA DEL CARGO ANTERIOR</x:v>
+      </x:c>
+      <x:c r="D58" s="90" t="str">
+        <x:v>CLAVE DEL CONCEPTO DE COBRO</x:v>
+      </x:c>
+      <x:c r="E58" s="90" t="str">
+        <x:v>NOMBRE DEL CONCEPTO DE COBRO</x:v>
+      </x:c>
+      <x:c r="F58" s="96" t="str">
+        <x:v>DESCRIPCIÓN DEL CARGO</x:v>
+      </x:c>
+      <x:c r="G58" s="96" t="str">
+        <x:v>FECHA DE EMISIÓN DEL CARGO</x:v>
+      </x:c>
+      <x:c r="H58" s="96" t="str">
+        <x:v>IMPORTE A APLICAR</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="24" customHeight="1">
+      <x:c r="A59" s="101" t="str">
+        <x:v>REF-2026-001</x:v>
+      </x:c>
+      <x:c r="B59" s="101" t="str">
+        <x:v>M-1001</x:v>
+      </x:c>
+      <x:c r="C59" s="101" t="str">
+        <x:v>CARGO-2026-1001</x:v>
+      </x:c>
+      <x:c r="D59" s="101" t="str">
+        <x:v>EJ-001</x:v>
+      </x:c>
+      <x:c r="E59" s="101" t="str">
+        <x:v>CUOTA DE MANTENIMIENTO</x:v>
+      </x:c>
+      <x:c r="F59" s="101" t="str">
+        <x:v>Registro de ejemplo para el socio 1001.</x:v>
+      </x:c>
+      <x:c r="G59" s="102" t="n">
+        <x:v>46037</x:v>
+      </x:c>
+      <x:c r="H59" s="103" t="n">
+        <x:v>2500</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="24" customHeight="1">
+      <x:c r="A60" s="101" t="str">
+        <x:v>REF-2026-002</x:v>
+      </x:c>
+      <x:c r="B60" s="101" t="str">
+        <x:v>M-1002</x:v>
+      </x:c>
+      <x:c r="C60" s="101" t="str">
+        <x:v>CARGO-2026-1002</x:v>
+      </x:c>
+      <x:c r="D60" s="101" t="str">
+        <x:v>EJ-002</x:v>
+      </x:c>
+      <x:c r="E60" s="101" t="str">
+        <x:v>CUOTA DE CASILLERO</x:v>
+      </x:c>
+      <x:c r="F60" s="101" t="str">
+        <x:v>Registro de ejemplo para el socio 1002.</x:v>
+      </x:c>
+      <x:c r="G60" s="102" t="n">
+        <x:v>46044.291666666664</x:v>
+      </x:c>
+      <x:c r="H60" s="103" t="n">
+        <x:v>850</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61" ht="24" customHeight="1">
+      <x:c r="A61" s="101" t="str">
+        <x:v>REF-2026-003</x:v>
+      </x:c>
+      <x:c r="B61" s="101" t="str">
+        <x:v>M-1003</x:v>
+      </x:c>
+      <x:c r="C61" s="101" t="str">
+        <x:v>CARGO-2026-1003</x:v>
+      </x:c>
+      <x:c r="D61" s="101" t="str">
+        <x:v>EJ-003</x:v>
+      </x:c>
+      <x:c r="E61" s="101" t="str">
+        <x:v>CLASE DE NATACIÓN</x:v>
+      </x:c>
+      <x:c r="F61" s="101" t="str">
+        <x:v>Registro de ejemplo para el socio 1003.</x:v>
+      </x:c>
+      <x:c r="G61" s="102" t="n">
+        <x:v>46051.333333333336</x:v>
+      </x:c>
+      <x:c r="H61" s="103" t="n">
+        <x:v>1200</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62" ht="42" customHeight="1">
+      <x:c r="A62"/>
+      <x:c r="B62"/>
+      <x:c r="C62"/>
+      <x:c r="D62"/>
+      <x:c r="E62"/>
+      <x:c r="F62"/>
+      <x:c r="G62"/>
+    </x:row>
+    <x:row r="63" ht="24" customHeight="1">
+      <x:c r="A63"/>
+      <x:c r="B63"/>
+      <x:c r="C63"/>
+      <x:c r="D63"/>
+      <x:c r="E63"/>
+      <x:c r="F63"/>
+      <x:c r="G63"/>
+    </x:row>
+    <x:row r="64" ht="24" customHeight="1">
+      <x:c r="A64" s="84" t="str">
+        <x:v>EJEMPLOS: FUENTES DE PAGO</x:v>
+      </x:c>
+      <x:c r="B64" s="84"/>
+      <x:c r="C64" s="84"/>
+      <x:c r="D64" s="84"/>
+      <x:c r="E64" s="84"/>
+      <x:c r="F64" s="84"/>
+      <x:c r="G64" s="84"/>
+      <x:c r="H64" s="84"/>
+      <x:c r="I64" s="84"/>
+      <x:c r="J64" s="84"/>
+      <x:c r="K64" s="84"/>
+      <x:c r="L64" s="84"/>
+      <x:c r="M64" s="84"/>
+      <x:c r="N64" s="84"/>
+    </x:row>
+    <x:row r="65" ht="42" customHeight="1">
+      <x:c r="A65" s="90" t="str">
+        <x:v>NÚMERO DE SOCIO</x:v>
+      </x:c>
+      <x:c r="B65" s="96" t="str">
+        <x:v>NOMBRE</x:v>
+      </x:c>
+      <x:c r="C65" s="96" t="str">
+        <x:v>APELLIDO PATERNO</x:v>
+      </x:c>
+      <x:c r="D65" s="96" t="str">
+        <x:v>APELLIDO MATERNO</x:v>
+      </x:c>
+      <x:c r="E65" s="90" t="str">
+        <x:v>NOMBRE DEL CLUB</x:v>
+      </x:c>
+      <x:c r="F65" s="96" t="str">
+        <x:v>IDENTIFICADOR DE LA TARJETA EN EL PROVEEDOR</x:v>
+      </x:c>
+      <x:c r="G65" s="96" t="str">
+        <x:v>TIPO DE TARJETA</x:v>
+      </x:c>
+      <x:c r="H65" s="96" t="str">
+        <x:v>ÚLTIMOS CUATRO DÍGITOS</x:v>
+      </x:c>
+      <x:c r="I65" s="96" t="str">
+        <x:v>MARCA DE LA TARJETA</x:v>
+      </x:c>
+      <x:c r="J65" s="96" t="str">
+        <x:v>MES DE VENCIMIENTO</x:v>
+      </x:c>
+      <x:c r="K65" s="96" t="str">
+        <x:v>AÑO DE VENCIMIENTO</x:v>
+      </x:c>
+      <x:c r="L65" s="96" t="str">
+        <x:v>NOMBRE DEL TITULAR DE LA TARJETA</x:v>
+      </x:c>
+      <x:c r="M65" s="96" t="str">
+        <x:v>ES LA TARJETA PREDETERMINADA</x:v>
+      </x:c>
+      <x:c r="N65" s="96" t="str">
+        <x:v>FECHA DE BAJA</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66" ht="24" customHeight="1">
+      <x:c r="A66" s="101" t="str">
+        <x:v>1001</x:v>
+      </x:c>
+      <x:c r="B66" s="101" t="str">
+        <x:v>Juan Carlos</x:v>
+      </x:c>
+      <x:c r="C66" s="101" t="str">
+        <x:v>Pérez</x:v>
+      </x:c>
+      <x:c r="D66" s="101" t="str">
+        <x:v>Hernández</x:v>
+      </x:c>
+      <x:c r="E66" s="101" t="str">
+        <x:v>PARQUE ESPAÑA</x:v>
+      </x:c>
+      <x:c r="F66" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 1</x:v>
+      </x:c>
+      <x:c r="G66" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 1</x:v>
+      </x:c>
+      <x:c r="H66" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 1</x:v>
+      </x:c>
+      <x:c r="I66" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 1</x:v>
+      </x:c>
+      <x:c r="J66" s="101" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K66" s="101" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="L66" s="101" t="str">
+        <x:v>SÍ</x:v>
+      </x:c>
+      <x:c r="M66" s="101" t="str">
+        <x:v>SÍ</x:v>
+      </x:c>
+      <x:c r="N66" s="102" t="n">
+        <x:v>46037</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67" ht="24" customHeight="1">
+      <x:c r="A67" s="101" t="str">
+        <x:v>1002</x:v>
+      </x:c>
+      <x:c r="B67" s="101" t="str">
+        <x:v>María Fernanda</x:v>
+      </x:c>
+      <x:c r="C67" s="101" t="str">
+        <x:v>López</x:v>
+      </x:c>
+      <x:c r="D67" s="101" t="str">
+        <x:v>García</x:v>
+      </x:c>
+      <x:c r="E67" s="101" t="str">
+        <x:v>PARQUE ESPAÑA</x:v>
+      </x:c>
+      <x:c r="F67" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 2</x:v>
+      </x:c>
+      <x:c r="G67" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 2</x:v>
+      </x:c>
+      <x:c r="H67" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 2</x:v>
+      </x:c>
+      <x:c r="I67" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 2</x:v>
+      </x:c>
+      <x:c r="J67" s="101" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="K67" s="101" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="L67" s="101" t="str">
+        <x:v>SÍ</x:v>
+      </x:c>
+      <x:c r="M67" s="101" t="str">
+        <x:v>SÍ</x:v>
+      </x:c>
+      <x:c r="N67" s="102" t="n">
+        <x:v>46044.291666666664</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="24" customHeight="1">
+      <x:c r="A68" s="101" t="str">
+        <x:v>1003</x:v>
+      </x:c>
+      <x:c r="B68" s="101" t="str">
+        <x:v>Roberto</x:v>
+      </x:c>
+      <x:c r="C68" s="101" t="str">
+        <x:v>Sánchez</x:v>
+      </x:c>
+      <x:c r="D68" s="101" t="str">
+        <x:v>Morales</x:v>
+      </x:c>
+      <x:c r="E68" s="101" t="str">
+        <x:v>PARQUE ESPAÑA</x:v>
+      </x:c>
+      <x:c r="F68" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 3</x:v>
+      </x:c>
+      <x:c r="G68" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 3</x:v>
+      </x:c>
+      <x:c r="H68" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 3</x:v>
+      </x:c>
+      <x:c r="I68" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 3</x:v>
+      </x:c>
+      <x:c r="J68" s="101" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="K68" s="101" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="L68" s="101" t="str">
+        <x:v>SÍ</x:v>
+      </x:c>
+      <x:c r="M68" s="101" t="str">
+        <x:v>SÍ</x:v>
+      </x:c>
+      <x:c r="N68" s="102" t="n">
+        <x:v>46051.333333333336</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="24" customHeight="1">
+      <x:c r="A71" s="84" t="str">
+        <x:v>EJEMPLOS: CORTES DE CAJA</x:v>
+      </x:c>
+      <x:c r="B71" s="84"/>
+      <x:c r="C71" s="84"/>
+      <x:c r="D71" s="84"/>
+      <x:c r="E71" s="84"/>
+      <x:c r="F71" s="84"/>
+      <x:c r="G71" s="84"/>
+      <x:c r="H71" s="84"/>
+      <x:c r="I71" s="84"/>
+      <x:c r="J71" s="84"/>
+      <x:c r="K71" s="84"/>
+      <x:c r="L71" s="84"/>
+      <x:c r="M71" s="84"/>
+      <x:c r="N71" s="84"/>
+    </x:row>
+    <x:row r="72" ht="42" customHeight="1">
+      <x:c r="A72" s="90" t="str">
+        <x:v>FOLIO O REFERENCIA DEL CORTE ANTERIOR</x:v>
+      </x:c>
+      <x:c r="B72" s="90" t="str">
+        <x:v>NOMBRE DEL CLUB</x:v>
+      </x:c>
+      <x:c r="C72" s="96" t="str">
+        <x:v>NOMBRE DEL CAJERO</x:v>
+      </x:c>
+      <x:c r="D72" s="96" t="str">
+        <x:v>CORREO DEL CAJERO</x:v>
+      </x:c>
+      <x:c r="E72" s="90" t="str">
+        <x:v>FECHA DEL CORTE</x:v>
+      </x:c>
+      <x:c r="F72" s="96" t="str">
+        <x:v>FONDO INICIAL</x:v>
+      </x:c>
+      <x:c r="G72" s="90" t="str">
+        <x:v>ESTATUS</x:v>
+      </x:c>
+      <x:c r="H72" s="96" t="str">
+        <x:v>FECHA Y HORA DE APERTURA</x:v>
+      </x:c>
+      <x:c r="I72" s="96" t="str">
+        <x:v>FECHA Y HORA DE CIERRE</x:v>
+      </x:c>
+      <x:c r="J72" s="96" t="str">
+        <x:v>EFECTIVO CONTADO</x:v>
+      </x:c>
+      <x:c r="K72" s="96" t="str">
+        <x:v>EFECTIVO ESPERADO</x:v>
+      </x:c>
+      <x:c r="L72" s="96" t="str">
+        <x:v>DIFERENCIA DE EFECTIVO</x:v>
+      </x:c>
+      <x:c r="M72" s="90" t="str">
+        <x:v>FOLIO O REFERENCIA DEL CORTE GLOBAL</x:v>
+      </x:c>
+      <x:c r="N72" s="96" t="str">
+        <x:v>NOTAS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="24" customHeight="1">
+      <x:c r="A73" s="101" t="str">
+        <x:v>REF-2026-001</x:v>
+      </x:c>
+      <x:c r="B73" s="101" t="str">
+        <x:v>PARQUE ESPAÑA</x:v>
+      </x:c>
+      <x:c r="C73" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 1</x:v>
+      </x:c>
+      <x:c r="D73" s="101" t="str">
+        <x:v>juan.perez@example.com</x:v>
+      </x:c>
+      <x:c r="E73" s="102" t="n">
+        <x:v>46037</x:v>
+      </x:c>
+      <x:c r="F73" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 1</x:v>
+      </x:c>
+      <x:c r="G73" s="101" t="str">
+        <x:v>ACTIVO</x:v>
+      </x:c>
+      <x:c r="H73" s="104" t="n">
+        <x:v>46037.625</x:v>
+      </x:c>
+      <x:c r="I73" s="104" t="n">
+        <x:v>46037.625</x:v>
+      </x:c>
+      <x:c r="J73" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 1</x:v>
+      </x:c>
+      <x:c r="K73" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 1</x:v>
+      </x:c>
+      <x:c r="L73" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 1</x:v>
+      </x:c>
+      <x:c r="M73" s="101" t="str">
+        <x:v>REF-2026-001</x:v>
+      </x:c>
+      <x:c r="N73" s="101" t="str">
+        <x:v>Registro de ejemplo para el socio 1001.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="24" customHeight="1">
+      <x:c r="A74" s="101" t="str">
+        <x:v>REF-2026-002</x:v>
+      </x:c>
+      <x:c r="B74" s="101" t="str">
+        <x:v>PARQUE ESPAÑA</x:v>
+      </x:c>
+      <x:c r="C74" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 2</x:v>
+      </x:c>
+      <x:c r="D74" s="101" t="str">
+        <x:v>maria.lopez@example.com</x:v>
+      </x:c>
+      <x:c r="E74" s="102" t="n">
+        <x:v>46044.291666666664</x:v>
+      </x:c>
+      <x:c r="F74" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 2</x:v>
+      </x:c>
+      <x:c r="G74" s="101" t="str">
+        <x:v>PENDIENTE</x:v>
+      </x:c>
+      <x:c r="H74" s="104" t="n">
+        <x:v>46044.666666666664</x:v>
+      </x:c>
+      <x:c r="I74" s="104" t="n">
+        <x:v>46044.666666666664</x:v>
+      </x:c>
+      <x:c r="J74" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 2</x:v>
+      </x:c>
+      <x:c r="K74" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 2</x:v>
+      </x:c>
+      <x:c r="L74" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 2</x:v>
+      </x:c>
+      <x:c r="M74" s="101" t="str">
+        <x:v>REF-2026-002</x:v>
+      </x:c>
+      <x:c r="N74" s="101" t="str">
+        <x:v>Registro de ejemplo para el socio 1002.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="24" customHeight="1">
+      <x:c r="A75" s="101" t="str">
+        <x:v>REF-2026-003</x:v>
+      </x:c>
+      <x:c r="B75" s="101" t="str">
+        <x:v>PARQUE ESPAÑA</x:v>
+      </x:c>
+      <x:c r="C75" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 3</x:v>
+      </x:c>
+      <x:c r="D75" s="101" t="str">
+        <x:v>roberto.sanchez@example.com</x:v>
+      </x:c>
+      <x:c r="E75" s="102" t="n">
+        <x:v>46051.333333333336</x:v>
+      </x:c>
+      <x:c r="F75" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 3</x:v>
+      </x:c>
+      <x:c r="G75" s="101" t="str">
+        <x:v>ACTIVO</x:v>
+      </x:c>
+      <x:c r="H75" s="104" t="n">
+        <x:v>46051.708333333336</x:v>
+      </x:c>
+      <x:c r="I75" s="104" t="n">
+        <x:v>46051.708333333336</x:v>
+      </x:c>
+      <x:c r="J75" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 3</x:v>
+      </x:c>
+      <x:c r="K75" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 3</x:v>
+      </x:c>
+      <x:c r="L75" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 3</x:v>
+      </x:c>
+      <x:c r="M75" s="101" t="str">
+        <x:v>REF-2026-003</x:v>
+      </x:c>
+      <x:c r="N75" s="101" t="str">
+        <x:v>Registro de ejemplo para el socio 1003.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78" ht="24" customHeight="1">
+      <x:c r="A78" s="84" t="str">
+        <x:v>EJEMPLOS: DESGLOSE DE EFECTIVO</x:v>
+      </x:c>
+      <x:c r="B78" s="84"/>
+      <x:c r="C78" s="84"/>
+      <x:c r="D78" s="84"/>
+      <x:c r="E78" s="84"/>
+      <x:c r="F78" s="84"/>
+      <x:c r="G78" s="84"/>
+    </x:row>
+    <x:row r="79" ht="42" customHeight="1">
+      <x:c r="A79" s="90" t="str">
+        <x:v>FOLIO O REFERENCIA DEL CORTE ANTERIOR</x:v>
+      </x:c>
+      <x:c r="B79" s="90" t="str">
+        <x:v>NOMBRE DEL CLUB</x:v>
+      </x:c>
+      <x:c r="C79" s="96" t="str">
+        <x:v>CORREO DEL CAJERO</x:v>
+      </x:c>
+      <x:c r="D79" s="96" t="str">
+        <x:v>FECHA Y HORA DE APERTURA</x:v>
+      </x:c>
+      <x:c r="E79" s="96" t="str">
+        <x:v>DENOMINACIÓN</x:v>
+      </x:c>
+      <x:c r="F79" s="96" t="str">
+        <x:v>CANTIDAD</x:v>
+      </x:c>
+      <x:c r="G79" s="96" t="str">
+        <x:v>SUBTOTAL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="24" customHeight="1">
+      <x:c r="A80" s="101" t="str">
+        <x:v>REF-2026-001</x:v>
+      </x:c>
+      <x:c r="B80" s="101" t="str">
+        <x:v>PARQUE ESPAÑA</x:v>
+      </x:c>
+      <x:c r="C80" s="101" t="str">
+        <x:v>juan.perez@example.com</x:v>
+      </x:c>
+      <x:c r="D80" s="104" t="n">
+        <x:v>46037.625</x:v>
+      </x:c>
+      <x:c r="E80" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 1</x:v>
+      </x:c>
+      <x:c r="F80" s="101" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G80" s="103" t="n">
+        <x:v>2500</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="24" customHeight="1">
+      <x:c r="A81" s="101" t="str">
+        <x:v>REF-2026-002</x:v>
+      </x:c>
+      <x:c r="B81" s="101" t="str">
+        <x:v>PARQUE ESPAÑA</x:v>
+      </x:c>
+      <x:c r="C81" s="101" t="str">
+        <x:v>maria.lopez@example.com</x:v>
+      </x:c>
+      <x:c r="D81" s="104" t="n">
+        <x:v>46044.666666666664</x:v>
+      </x:c>
+      <x:c r="E81" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 2</x:v>
+      </x:c>
+      <x:c r="F81" s="101" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G81" s="103" t="n">
+        <x:v>850</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="24" customHeight="1">
+      <x:c r="A82" s="101" t="str">
+        <x:v>REF-2026-003</x:v>
+      </x:c>
+      <x:c r="B82" s="101" t="str">
+        <x:v>PARQUE ESPAÑA</x:v>
+      </x:c>
+      <x:c r="C82" s="101" t="str">
+        <x:v>roberto.sanchez@example.com</x:v>
+      </x:c>
+      <x:c r="D82" s="104" t="n">
+        <x:v>46051.708333333336</x:v>
+      </x:c>
+      <x:c r="E82" s="101" t="str">
+        <x:v>DATOS DE EJEMPLO 3</x:v>
+      </x:c>
+      <x:c r="F82" s="101" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G82" s="103" t="n">
+        <x:v>1200</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85" ht="24" customHeight="1">
+      <x:c r="A85" s="84" t="str">
+        <x:v>EJEMPLOS: CORTES GLOBALES</x:v>
+      </x:c>
+      <x:c r="B85" s="84"/>
+      <x:c r="C85" s="84"/>
+      <x:c r="D85" s="84"/>
+      <x:c r="E85" s="84"/>
+      <x:c r="F85" s="84"/>
+      <x:c r="G85" s="84"/>
+    </x:row>
+    <x:row r="86" ht="42" customHeight="1">
+      <x:c r="A86" s="90" t="str">
+        <x:v>FOLIO O REFERENCIA DEL CORTE GLOBAL</x:v>
+      </x:c>
+      <x:c r="B86" s="90" t="str">
+        <x:v>NOMBRE DEL CLUB</x:v>
+      </x:c>
+      <x:c r="C86" s="90" t="str">
+        <x:v>FECHA DEL CORTE</x:v>
+      </x:c>
+      <x:c r="D86" s="90" t="str">
+        <x:v>ESTATUS</x:v>
+      </x:c>
+      <x:c r="E86" s="96" t="str">
+        <x:v>CORREO DE QUIEN CREÓ EL CORTE</x:v>
+      </x:c>
+      <x:c r="F86" s="96" t="str">
+        <x:v>FECHA Y HORA DE CIERRE</x:v>
+      </x:c>
+      <x:c r="G86" s="96" t="str">
+        <x:v>NOTAS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87" ht="24" customHeight="1">
+      <x:c r="A87" s="101" t="str">
+        <x:v>REF-2026-001</x:v>
+      </x:c>
+      <x:c r="B87" s="101" t="str">
+        <x:v>PARQUE ESPAÑA</x:v>
+      </x:c>
+      <x:c r="C87" s="102" t="n">
+        <x:v>46037</x:v>
+      </x:c>
+      <x:c r="D87" s="101" t="str">
+        <x:v>ACTIVO</x:v>
+      </x:c>
+      <x:c r="E87" s="101" t="str">
+        <x:v>juan.perez@example.com</x:v>
+      </x:c>
+      <x:c r="F87" s="104" t="n">
+        <x:v>46037.625</x:v>
+      </x:c>
+      <x:c r="G87" s="101" t="str">
+        <x:v>Registro de ejemplo para el socio 1001.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="24" customHeight="1">
+      <x:c r="A88" s="101" t="str">
+        <x:v>REF-2026-002</x:v>
+      </x:c>
+      <x:c r="B88" s="101" t="str">
+        <x:v>PARQUE ESPAÑA</x:v>
+      </x:c>
+      <x:c r="C88" s="102" t="n">
+        <x:v>46044.291666666664</x:v>
+      </x:c>
+      <x:c r="D88" s="101" t="str">
+        <x:v>PENDIENTE</x:v>
+      </x:c>
+      <x:c r="E88" s="101" t="str">
+        <x:v>maria.lopez@example.com</x:v>
+      </x:c>
+      <x:c r="F88" s="104" t="n">
+        <x:v>46044.666666666664</x:v>
+      </x:c>
+      <x:c r="G88" s="101" t="str">
+        <x:v>Registro de ejemplo para el socio 1002.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="24" customHeight="1">
+      <x:c r="A89" s="101" t="str">
+        <x:v>REF-2026-003</x:v>
+      </x:c>
+      <x:c r="B89" s="101" t="str">
+        <x:v>PARQUE ESPAÑA</x:v>
+      </x:c>
+      <x:c r="C89" s="102" t="n">
+        <x:v>46051.333333333336</x:v>
+      </x:c>
+      <x:c r="D89" s="101" t="str">
+        <x:v>ACTIVO</x:v>
+      </x:c>
+      <x:c r="E89" s="101" t="str">
+        <x:v>roberto.sanchez@example.com</x:v>
+      </x:c>
+      <x:c r="F89" s="104" t="n">
+        <x:v>46051.708333333336</x:v>
+      </x:c>
+      <x:c r="G89" s="101" t="str">
+        <x:v>Registro de ejemplo para el socio 1003.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:G1"/>
+    <x:mergeCell ref="A8:V8"/>
+    <x:mergeCell ref="A15:T15"/>
+    <x:mergeCell ref="A22:L22"/>
+    <x:mergeCell ref="A29:D29"/>
+    <x:mergeCell ref="A36:H36"/>
+    <x:mergeCell ref="A43:E43"/>
+    <x:mergeCell ref="A50:M50"/>
+    <x:mergeCell ref="A57:H57"/>
+    <x:mergeCell ref="A64:N64"/>
+    <x:mergeCell ref="A71:N71"/>
+    <x:mergeCell ref="A78:G78"/>
+    <x:mergeCell ref="A85:G85"/>
+  </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -12340,70 +15039,70 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
-      <x:c r="A1" s="6" t="str">
+      <x:c r="A1" s="10" t="str">
         <x:v>FOLIO O REFERENCIA DEL CARGO ANTERIOR</x:v>
       </x:c>
-      <x:c r="B1" s="6" t="str">
+      <x:c r="B1" s="10" t="str">
         <x:v>NÚMERO DE MEMBRESÍA</x:v>
       </x:c>
-      <x:c r="C1" s="6" t="str">
+      <x:c r="C1" s="10" t="str">
         <x:v>NOMBRE DEL CLUB</x:v>
       </x:c>
-      <x:c r="D1" s="6" t="str">
+      <x:c r="D1" s="10" t="str">
         <x:v>NÚMERO DE SOCIO</x:v>
       </x:c>
-      <x:c r="E1" s="6" t="str">
+      <x:c r="E1" s="12" t="str">
         <x:v>NOMBRE</x:v>
       </x:c>
-      <x:c r="F1" s="6" t="str">
+      <x:c r="F1" s="12" t="str">
         <x:v>APELLIDO PATERNO</x:v>
       </x:c>
-      <x:c r="G1" s="6" t="str">
+      <x:c r="G1" s="12" t="str">
         <x:v>APELLIDO MATERNO</x:v>
       </x:c>
-      <x:c r="H1" s="6" t="str">
+      <x:c r="H1" s="12" t="str">
         <x:v>TIPO DE MEMBRESÍA</x:v>
       </x:c>
-      <x:c r="I1" s="6" t="str">
+      <x:c r="I1" s="10" t="str">
         <x:v>CLAVE DEL CONCEPTO DE COBRO</x:v>
       </x:c>
-      <x:c r="J1" s="6" t="str">
+      <x:c r="J1" s="10" t="str">
         <x:v>NOMBRE DEL CONCEPTO DE COBRO</x:v>
       </x:c>
-      <x:c r="K1" s="6" t="str">
+      <x:c r="K1" s="12" t="str">
         <x:v>DESCRIPCIÓN DEL CARGO</x:v>
       </x:c>
-      <x:c r="L1" s="6" t="str">
+      <x:c r="L1" s="12" t="str">
         <x:v>IMPORTE ORIGINAL</x:v>
       </x:c>
-      <x:c r="M1" s="6" t="str">
+      <x:c r="M1" s="12" t="str">
         <x:v>SALDO PENDIENTE</x:v>
       </x:c>
-      <x:c r="N1" s="6" t="str">
+      <x:c r="N1" s="12" t="str">
         <x:v>FECHA DE EMISIÓN</x:v>
       </x:c>
-      <x:c r="O1" s="6" t="str">
+      <x:c r="O1" s="12" t="str">
         <x:v>FECHA DE VENCIMIENTO</x:v>
       </x:c>
-      <x:c r="P1" s="6" t="str">
+      <x:c r="P1" s="12" t="str">
         <x:v>AÑO DEL PERIODO</x:v>
       </x:c>
-      <x:c r="Q1" s="6" t="str">
+      <x:c r="Q1" s="12" t="str">
         <x:v>MES DEL PERIODO</x:v>
       </x:c>
-      <x:c r="R1" s="6" t="str">
+      <x:c r="R1" s="12" t="str">
         <x:v>PERMITE ABONOS</x:v>
       </x:c>
-      <x:c r="S1" s="6" t="str">
+      <x:c r="S1" s="10" t="str">
         <x:v>ESTATUS</x:v>
       </x:c>
-      <x:c r="T1" s="6" t="str">
+      <x:c r="T1" s="12" t="str">
         <x:v>FECHA DE CANCELACIÓN</x:v>
       </x:c>
-      <x:c r="U1" s="6" t="str">
+      <x:c r="U1" s="12" t="str">
         <x:v>CORREO DE QUIEN CANCELÓ</x:v>
       </x:c>
-      <x:c r="V1" s="6" t="str">
+      <x:c r="V1" s="12" t="str">
         <x:v>MOTIVO DE CANCELACIÓN</x:v>
       </x:c>
     </x:row>
@@ -17218,64 +19917,64 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
-      <x:c r="A1" s="6" t="str">
+      <x:c r="A1" s="10" t="str">
         <x:v>FOLIO O REFERENCIA DEL PAGO ANTERIOR</x:v>
       </x:c>
-      <x:c r="B1" s="6" t="str">
+      <x:c r="B1" s="12" t="str">
         <x:v>FOLIO DEL COMPROBANTE</x:v>
       </x:c>
-      <x:c r="C1" s="6" t="str">
+      <x:c r="C1" s="10" t="str">
         <x:v>NÚMERO DE MEMBRESÍA</x:v>
       </x:c>
-      <x:c r="D1" s="6" t="str">
+      <x:c r="D1" s="10" t="str">
         <x:v>NOMBRE DEL CLUB</x:v>
       </x:c>
-      <x:c r="E1" s="6" t="str">
+      <x:c r="E1" s="12" t="str">
         <x:v>MÉTODO DE PAGO</x:v>
       </x:c>
-      <x:c r="F1" s="6" t="str">
+      <x:c r="F1" s="12" t="str">
         <x:v>IMPORTE PAGADO</x:v>
       </x:c>
-      <x:c r="G1" s="6" t="str">
+      <x:c r="G1" s="12" t="str">
         <x:v>SUBTOTAL</x:v>
       </x:c>
-      <x:c r="H1" s="6" t="str">
+      <x:c r="H1" s="12" t="str">
         <x:v>IVA</x:v>
       </x:c>
-      <x:c r="I1" s="6" t="str">
+      <x:c r="I1" s="12" t="str">
         <x:v>FECHA Y HORA DEL PAGO</x:v>
       </x:c>
-      <x:c r="J1" s="6" t="str">
+      <x:c r="J1" s="12" t="str">
         <x:v>REFERENCIA BANCARIA</x:v>
       </x:c>
-      <x:c r="K1" s="6" t="str">
+      <x:c r="K1" s="12" t="str">
         <x:v>NOMBRE DEL BANCO</x:v>
       </x:c>
-      <x:c r="L1" s="6" t="str">
+      <x:c r="L1" s="12" t="str">
         <x:v>NÚMERO DE CHEQUE</x:v>
       </x:c>
-      <x:c r="M1" s="6" t="str">
+      <x:c r="M1" s="12" t="str">
         <x:v>NOTAS</x:v>
       </x:c>
-      <x:c r="N1" s="6" t="str">
+      <x:c r="N1" s="12" t="str">
         <x:v>CORREO DE QUIEN RECIBIÓ</x:v>
       </x:c>
-      <x:c r="O1" s="6" t="str">
+      <x:c r="O1" s="10" t="str">
         <x:v>ESTATUS</x:v>
       </x:c>
-      <x:c r="P1" s="6" t="str">
+      <x:c r="P1" s="12" t="str">
         <x:v>NOMBRE DEL ARCHIVO DEL COMPROBANTE</x:v>
       </x:c>
-      <x:c r="Q1" s="6" t="str">
+      <x:c r="Q1" s="12" t="str">
         <x:v>REFERENCIA DE LA OPERACIÓN AGRUPADA</x:v>
       </x:c>
-      <x:c r="R1" s="6" t="str">
+      <x:c r="R1" s="12" t="str">
         <x:v>FECHA DE CANCELACIÓN</x:v>
       </x:c>
-      <x:c r="S1" s="6" t="str">
+      <x:c r="S1" s="12" t="str">
         <x:v>CORREO DE QUIEN CANCELÓ</x:v>
       </x:c>
-      <x:c r="T1" s="6" t="str">
+      <x:c r="T1" s="12" t="str">
         <x:v>MOTIVO DE CANCELACIÓN</x:v>
       </x:c>
     </x:row>
@@ -21684,40 +24383,40 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
-      <x:c r="A1" s="6" t="str">
+      <x:c r="A1" s="10" t="str">
         <x:v>FOLIO O REFERENCIA DEL PAGO ANTERIOR</x:v>
       </x:c>
-      <x:c r="B1" s="6" t="str">
+      <x:c r="B1" s="12" t="str">
         <x:v>FOLIO DEL COMPROBANTE</x:v>
       </x:c>
-      <x:c r="C1" s="6" t="str">
+      <x:c r="C1" s="10" t="str">
         <x:v>FOLIO O REFERENCIA DEL CARGO ANTERIOR</x:v>
       </x:c>
-      <x:c r="D1" s="6" t="str">
+      <x:c r="D1" s="10" t="str">
         <x:v>NÚMERO DE MEMBRESÍA</x:v>
       </x:c>
-      <x:c r="E1" s="6" t="str">
+      <x:c r="E1" s="10" t="str">
         <x:v>CLAVE DEL CONCEPTO DE COBRO</x:v>
       </x:c>
-      <x:c r="F1" s="6" t="str">
+      <x:c r="F1" s="10" t="str">
         <x:v>NOMBRE DEL CONCEPTO DE COBRO</x:v>
       </x:c>
-      <x:c r="G1" s="6" t="str">
+      <x:c r="G1" s="12" t="str">
         <x:v>DESCRIPCIÓN DEL CARGO</x:v>
       </x:c>
-      <x:c r="H1" s="6" t="str">
+      <x:c r="H1" s="12" t="str">
         <x:v>FECHA DE EMISIÓN DEL CARGO</x:v>
       </x:c>
-      <x:c r="I1" s="6" t="str">
+      <x:c r="I1" s="12" t="str">
         <x:v>IMPORTE APLICADO</x:v>
       </x:c>
-      <x:c r="J1" s="6" t="str">
+      <x:c r="J1" s="12" t="str">
         <x:v>SUBTOTAL APLICADO</x:v>
       </x:c>
-      <x:c r="K1" s="6" t="str">
+      <x:c r="K1" s="12" t="str">
         <x:v>IVA APLICADO</x:v>
       </x:c>
-      <x:c r="L1" s="6" t="str">
+      <x:c r="L1" s="12" t="str">
         <x:v>DESCUENTO APLICADO</x:v>
       </x:c>
     </x:row>
@@ -24526,16 +27225,16 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
-      <x:c r="A1" s="6" t="str">
+      <x:c r="A1" s="10" t="str">
         <x:v>NÚMERO DE MEMBRESÍA</x:v>
       </x:c>
-      <x:c r="B1" s="6" t="str">
+      <x:c r="B1" s="10" t="str">
         <x:v>NOMBRE DEL CLUB</x:v>
       </x:c>
-      <x:c r="C1" s="6" t="str">
+      <x:c r="C1" s="12" t="str">
         <x:v>IMPORTE DEL SALDO A FAVOR</x:v>
       </x:c>
-      <x:c r="D1" s="6" t="str">
+      <x:c r="D1" s="12" t="str">
         <x:v>FECHA DE CORTE</x:v>
       </x:c>
     </x:row>
@@ -25756,28 +28455,28 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
-      <x:c r="A1" s="6" t="str">
+      <x:c r="A1" s="10" t="str">
         <x:v>NÚMERO DE MEMBRESÍA</x:v>
       </x:c>
-      <x:c r="B1" s="6" t="str">
+      <x:c r="B1" s="10" t="str">
         <x:v>NOMBRE DEL CLUB</x:v>
       </x:c>
-      <x:c r="C1" s="6" t="str">
+      <x:c r="C1" s="12" t="str">
         <x:v>FECHA Y HORA DEL MOVIMIENTO</x:v>
       </x:c>
-      <x:c r="D1" s="6" t="str">
+      <x:c r="D1" s="12" t="str">
         <x:v>IMPORTE DEL MOVIMIENTO</x:v>
       </x:c>
-      <x:c r="E1" s="6" t="str">
+      <x:c r="E1" s="12" t="str">
         <x:v>CONCEPTO DEL MOVIMIENTO</x:v>
       </x:c>
-      <x:c r="F1" s="6" t="str">
+      <x:c r="F1" s="10" t="str">
         <x:v>FOLIO O REFERENCIA DEL CARGO ANTERIOR</x:v>
       </x:c>
-      <x:c r="G1" s="6" t="str">
+      <x:c r="G1" s="10" t="str">
         <x:v>FOLIO O REFERENCIA DEL PAGO ANTERIOR</x:v>
       </x:c>
-      <x:c r="H1" s="6" t="str">
+      <x:c r="H1" s="12" t="str">
         <x:v>NOTAS</x:v>
       </x:c>
     </x:row>
@@ -27791,19 +30490,19 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
-      <x:c r="A1" s="6" t="str">
+      <x:c r="A1" s="10" t="str">
         <x:v>NÚMERO DE MEMBRESÍA</x:v>
       </x:c>
-      <x:c r="B1" s="6" t="str">
+      <x:c r="B1" s="10" t="str">
         <x:v>NOMBRE DEL CLUB</x:v>
       </x:c>
-      <x:c r="C1" s="6" t="str">
+      <x:c r="C1" s="12" t="str">
         <x:v>FECHA Y HORA DE LA NOTA</x:v>
       </x:c>
-      <x:c r="D1" s="6" t="str">
+      <x:c r="D1" s="12" t="str">
         <x:v>CORREO DE QUIEN REGISTRÓ LA NOTA</x:v>
       </x:c>
-      <x:c r="E1" s="6" t="str">
+      <x:c r="E1" s="12" t="str">
         <x:v>NOTA DE COBRANZA</x:v>
       </x:c>
     </x:row>
@@ -29228,43 +31927,43 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
-      <x:c r="A1" s="6" t="str">
+      <x:c r="A1" s="10" t="str">
         <x:v>FOLIO O REFERENCIA DE LA OPERACIÓN ANTERIOR</x:v>
       </x:c>
-      <x:c r="B1" s="6" t="str">
+      <x:c r="B1" s="10" t="str">
         <x:v>NÚMERO DE MEMBRESÍA</x:v>
       </x:c>
-      <x:c r="C1" s="6" t="str">
+      <x:c r="C1" s="10" t="str">
         <x:v>NOMBRE DEL CLUB</x:v>
       </x:c>
-      <x:c r="D1" s="6" t="str">
+      <x:c r="D1" s="12" t="str">
         <x:v>MÉTODO DE PAGO</x:v>
       </x:c>
-      <x:c r="E1" s="6" t="str">
+      <x:c r="E1" s="12" t="str">
         <x:v>FOLIO DE LA ORDEN EN EL PROVEEDOR</x:v>
       </x:c>
-      <x:c r="F1" s="6" t="str">
+      <x:c r="F1" s="12" t="str">
         <x:v>FOLIO DEL CARGO EN EL PROVEEDOR</x:v>
       </x:c>
-      <x:c r="G1" s="6" t="str">
+      <x:c r="G1" s="12" t="str">
         <x:v>CLABE</x:v>
       </x:c>
-      <x:c r="H1" s="6" t="str">
+      <x:c r="H1" s="12" t="str">
         <x:v>NOMBRE DEL BANCO</x:v>
       </x:c>
-      <x:c r="I1" s="6" t="str">
+      <x:c r="I1" s="12" t="str">
         <x:v>IMPORTE</x:v>
       </x:c>
-      <x:c r="J1" s="6" t="str">
+      <x:c r="J1" s="12" t="str">
         <x:v>FECHA Y HORA DE VENCIMIENTO</x:v>
       </x:c>
-      <x:c r="K1" s="6" t="str">
+      <x:c r="K1" s="10" t="str">
         <x:v>ESTATUS</x:v>
       </x:c>
-      <x:c r="L1" s="6" t="str">
+      <x:c r="L1" s="10" t="str">
         <x:v>FOLIO O REFERENCIA DEL PAGO ANTERIOR</x:v>
       </x:c>
-      <x:c r="M1" s="6" t="str">
+      <x:c r="M1" s="12" t="str">
         <x:v>NOTAS</x:v>
       </x:c>
     </x:row>
@@ -32276,28 +34975,28 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
-      <x:c r="A1" s="6" t="str">
+      <x:c r="A1" s="10" t="str">
         <x:v>FOLIO O REFERENCIA DE LA OPERACIÓN ANTERIOR</x:v>
       </x:c>
-      <x:c r="B1" s="6" t="str">
+      <x:c r="B1" s="10" t="str">
         <x:v>NÚMERO DE MEMBRESÍA</x:v>
       </x:c>
-      <x:c r="C1" s="6" t="str">
+      <x:c r="C1" s="10" t="str">
         <x:v>FOLIO O REFERENCIA DEL CARGO ANTERIOR</x:v>
       </x:c>
-      <x:c r="D1" s="6" t="str">
+      <x:c r="D1" s="10" t="str">
         <x:v>CLAVE DEL CONCEPTO DE COBRO</x:v>
       </x:c>
-      <x:c r="E1" s="6" t="str">
+      <x:c r="E1" s="10" t="str">
         <x:v>NOMBRE DEL CONCEPTO DE COBRO</x:v>
       </x:c>
-      <x:c r="F1" s="6" t="str">
+      <x:c r="F1" s="12" t="str">
         <x:v>DESCRIPCIÓN DEL CARGO</x:v>
       </x:c>
-      <x:c r="G1" s="6" t="str">
+      <x:c r="G1" s="12" t="str">
         <x:v>FECHA DE EMISIÓN DEL CARGO</x:v>
       </x:c>
-      <x:c r="H1" s="6" t="str">
+      <x:c r="H1" s="12" t="str">
         <x:v>IMPORTE A APLICAR</x:v>
       </x:c>
     </x:row>

</xml_diff>